<commit_message>
Full enrichment of all 208 schools, re-scored exports, handoff doc
--all run: 133 schools with NCES district and enrollment, 76 with a
website, 22 band pages, 5 booster clubs, 3 labelled director names,
1 labelled director email; 60 rows have no NCES website, 20 school
sites blocked the crawler, 41 rows have no state. Nickname text is no
longer kept as a city at merge time. docs/HANDOFF.md documents the
project, decisions, data model, source status, gaps, and next steps.

Co-Authored-By: Claude Fable 5.1 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_014hr17qS7ZCdG5VTCbF27VQ
</commit_message>
<xml_diff>
--- a/data/final/prospects.xlsx
+++ b/data/final/prospects.xlsx
@@ -734,12 +734,12 @@
       </c>
       <c r="D4" t="inlineStr">
         <is>
-          <t>The Pride of</t>
+          <t>The Pride of Broken Arrow</t>
         </is>
       </c>
       <c r="E4" t="inlineStr">
         <is>
-          <t>The Pride of Broken Arrow</t>
+          <t>Broken Arrow</t>
         </is>
       </c>
       <c r="F4" t="inlineStr">
@@ -3186,7 +3186,7 @@
       </c>
       <c r="E38" t="inlineStr">
         <is>
-          <t>Red Raider Marching Band</t>
+          <t>Pulaski</t>
         </is>
       </c>
       <c r="F38" t="inlineStr">
@@ -6317,20 +6317,43 @@
         <v>2019</v>
       </c>
       <c r="J36" t="inlineStr"/>
-      <c r="K36" t="inlineStr"/>
-      <c r="L36" t="inlineStr"/>
-      <c r="M36" t="inlineStr"/>
-      <c r="N36" t="inlineStr"/>
+      <c r="K36" t="inlineStr">
+        <is>
+          <t>Cobb County</t>
+        </is>
+      </c>
+      <c r="L36" t="n">
+        <v>1949</v>
+      </c>
+      <c r="M36" t="inlineStr">
+        <is>
+          <t>http://www.cobbk12.org/lassiter</t>
+        </is>
+      </c>
+      <c r="N36" t="inlineStr">
+        <is>
+          <t>http://www.cobbk12.org/lassiter/band</t>
+        </is>
+      </c>
       <c r="O36" t="inlineStr"/>
       <c r="P36" t="inlineStr"/>
       <c r="Q36" t="inlineStr"/>
-      <c r="R36" t="inlineStr"/>
+      <c r="R36" t="inlineStr">
+        <is>
+          <t>Our supportive parent community and Lassiter Band Booster Association raise funds that</t>
+        </is>
+      </c>
       <c r="S36" s="2" t="inlineStr">
         <is>
-          <t>https://en.wikipedia.org/wiki/Rose_Parade_marching_bands</t>
-        </is>
-      </c>
-      <c r="T36" s="2" t="inlineStr"/>
+          <t>https://en.wikipedia.org/wiki/Rose_Parade_marching_bands
+http://www.cobbk12.org/lassiter/band</t>
+        </is>
+      </c>
+      <c r="T36" s="2" t="inlineStr">
+        <is>
+          <t>social: https://www.facebook.com/cobbschools</t>
+        </is>
+      </c>
     </row>
     <row r="37">
       <c r="A37" t="inlineStr">
@@ -6449,9 +6472,19 @@
         <v>2019</v>
       </c>
       <c r="J38" t="inlineStr"/>
-      <c r="K38" t="inlineStr"/>
-      <c r="L38" t="inlineStr"/>
-      <c r="M38" t="inlineStr"/>
+      <c r="K38" t="inlineStr">
+        <is>
+          <t>Tipton County</t>
+        </is>
+      </c>
+      <c r="L38" t="n">
+        <v>1273</v>
+      </c>
+      <c r="M38" t="inlineStr">
+        <is>
+          <t>http://www.tipton-county.com/mhs</t>
+        </is>
+      </c>
       <c r="N38" t="inlineStr"/>
       <c r="O38" t="inlineStr"/>
       <c r="P38" t="inlineStr"/>
@@ -6462,7 +6495,11 @@
           <t>https://en.wikipedia.org/wiki/Rose_Parade_marching_bands</t>
         </is>
       </c>
-      <c r="T38" s="2" t="inlineStr"/>
+      <c r="T38" s="2" t="inlineStr">
+        <is>
+          <t>site crawl blocked: HTTP 403 / challenge page for http://www.tipton-county.com/mhs</t>
+        </is>
+      </c>
     </row>
     <row r="39">
       <c r="A39" t="inlineStr">
@@ -6549,9 +6586,19 @@
         <v>2017</v>
       </c>
       <c r="J40" t="inlineStr"/>
-      <c r="K40" t="inlineStr"/>
-      <c r="L40" t="inlineStr"/>
-      <c r="M40" t="inlineStr"/>
+      <c r="K40" t="inlineStr">
+        <is>
+          <t>Hamilton County</t>
+        </is>
+      </c>
+      <c r="L40" t="n">
+        <v>1275</v>
+      </c>
+      <c r="M40" t="inlineStr">
+        <is>
+          <t>http://ohs.hcde.org/</t>
+        </is>
+      </c>
       <c r="N40" t="inlineStr"/>
       <c r="O40" t="inlineStr"/>
       <c r="P40" t="inlineStr"/>
@@ -6562,7 +6609,11 @@
           <t>https://en.wikipedia.org/wiki/Rose_Parade_marching_bands</t>
         </is>
       </c>
-      <c r="T40" s="2" t="inlineStr"/>
+      <c r="T40" s="2" t="inlineStr">
+        <is>
+          <t>no band page found in 2 pages crawled</t>
+        </is>
+      </c>
     </row>
     <row r="41">
       <c r="A41" t="inlineStr">
@@ -6939,9 +6990,19 @@
         <v>2015</v>
       </c>
       <c r="J46" t="inlineStr"/>
-      <c r="K46" t="inlineStr"/>
-      <c r="L46" t="inlineStr"/>
-      <c r="M46" t="inlineStr"/>
+      <c r="K46" t="inlineStr">
+        <is>
+          <t>Cobb County</t>
+        </is>
+      </c>
+      <c r="L46" t="n">
+        <v>2685</v>
+      </c>
+      <c r="M46" t="inlineStr">
+        <is>
+          <t>http://www.waltonhigh.org</t>
+        </is>
+      </c>
       <c r="N46" t="inlineStr"/>
       <c r="O46" t="inlineStr"/>
       <c r="P46" t="inlineStr"/>
@@ -6952,7 +7013,11 @@
           <t>https://en.wikipedia.org/wiki/Rose_Parade_marching_bands</t>
         </is>
       </c>
-      <c r="T46" s="2" t="inlineStr"/>
+      <c r="T46" s="2" t="inlineStr">
+        <is>
+          <t>no band page found in 1 pages crawled</t>
+        </is>
+      </c>
     </row>
     <row r="47">
       <c r="A47" t="inlineStr">
@@ -7150,7 +7215,7 @@
       </c>
       <c r="T49" s="2" t="inlineStr">
         <is>
-          <t>state unknown: source lists no location</t>
+          <t>state unknown: source lists no location; nces: skipped (state unknown)</t>
         </is>
       </c>
     </row>
@@ -7202,7 +7267,7 @@
       </c>
       <c r="T50" s="2" t="inlineStr">
         <is>
-          <t>state unknown: source lists no location</t>
+          <t>state unknown: source lists no location; nces: skipped (state unknown)</t>
         </is>
       </c>
     </row>
@@ -7316,7 +7381,11 @@
           <t>https://en.wikipedia.org/wiki/Rose_Parade_marching_bands</t>
         </is>
       </c>
-      <c r="T52" s="2" t="inlineStr"/>
+      <c r="T52" s="2" t="inlineStr">
+        <is>
+          <t>nces: no match</t>
+        </is>
+      </c>
     </row>
     <row r="53">
       <c r="A53" t="inlineStr">
@@ -7424,7 +7493,11 @@
           <t>https://en.wikipedia.org/wiki/Rose_Parade_marching_bands</t>
         </is>
       </c>
-      <c r="T54" s="2" t="inlineStr"/>
+      <c r="T54" s="2" t="inlineStr">
+        <is>
+          <t>nces: no match</t>
+        </is>
+      </c>
     </row>
     <row r="55">
       <c r="A55" t="inlineStr">
@@ -7467,9 +7540,19 @@
         <v>2020</v>
       </c>
       <c r="J55" t="inlineStr"/>
-      <c r="K55" t="inlineStr"/>
-      <c r="L55" t="inlineStr"/>
-      <c r="M55" t="inlineStr"/>
+      <c r="K55" t="inlineStr">
+        <is>
+          <t>HARRISON CO SCHOOL DIST</t>
+        </is>
+      </c>
+      <c r="L55" t="n">
+        <v>1154</v>
+      </c>
+      <c r="M55" t="inlineStr">
+        <is>
+          <t>http://www.harrison.k12.ms.us/home/westharrisonhigh.aspx</t>
+        </is>
+      </c>
       <c r="N55" t="inlineStr"/>
       <c r="O55" t="inlineStr"/>
       <c r="P55" t="inlineStr"/>
@@ -7480,7 +7563,11 @@
           <t>https://en.wikipedia.org/wiki/Rose_Parade_marching_bands</t>
         </is>
       </c>
-      <c r="T55" s="2" t="inlineStr"/>
+      <c r="T55" s="2" t="inlineStr">
+        <is>
+          <t>no band page found in 1 pages crawled</t>
+        </is>
+      </c>
     </row>
     <row r="56">
       <c r="A56" t="inlineStr">
@@ -7519,8 +7606,14 @@
         <v>2017</v>
       </c>
       <c r="J56" t="inlineStr"/>
-      <c r="K56" t="inlineStr"/>
-      <c r="L56" t="inlineStr"/>
+      <c r="K56" t="inlineStr">
+        <is>
+          <t>EANES ISD</t>
+        </is>
+      </c>
+      <c r="L56" t="n">
+        <v>2811</v>
+      </c>
       <c r="M56" t="inlineStr"/>
       <c r="N56" t="inlineStr"/>
       <c r="O56" t="inlineStr"/>
@@ -7532,7 +7625,11 @@
           <t>https://en.wikipedia.org/wiki/Rose_Parade_marching_bands</t>
         </is>
       </c>
-      <c r="T56" s="2" t="inlineStr"/>
+      <c r="T56" s="2" t="inlineStr">
+        <is>
+          <t>no website in NCES</t>
+        </is>
+      </c>
     </row>
     <row r="57">
       <c r="A57" t="inlineStr">
@@ -7646,7 +7743,7 @@
       </c>
       <c r="T58" s="2" t="inlineStr">
         <is>
-          <t>state unknown: source lists no location</t>
+          <t>state unknown: source lists no location; nces: skipped (state unknown)</t>
         </is>
       </c>
     </row>
@@ -7691,8 +7788,14 @@
         <v>2018</v>
       </c>
       <c r="J59" t="inlineStr"/>
-      <c r="K59" t="inlineStr"/>
-      <c r="L59" t="inlineStr"/>
+      <c r="K59" t="inlineStr">
+        <is>
+          <t>Academy School District No. 20 in the county of El Paso an</t>
+        </is>
+      </c>
+      <c r="L59" t="n">
+        <v>1315</v>
+      </c>
       <c r="M59" t="inlineStr"/>
       <c r="N59" t="inlineStr"/>
       <c r="O59" t="inlineStr"/>
@@ -7704,7 +7807,11 @@
           <t>https://en.wikipedia.org/wiki/Rose_Parade_marching_bands</t>
         </is>
       </c>
-      <c r="T59" s="2" t="inlineStr"/>
+      <c r="T59" s="2" t="inlineStr">
+        <is>
+          <t>no website in NCES</t>
+        </is>
+      </c>
     </row>
     <row r="60">
       <c r="A60" t="inlineStr">
@@ -7760,7 +7867,11 @@
           <t>https://en.wikipedia.org/wiki/Rose_Parade_marching_bands</t>
         </is>
       </c>
-      <c r="T60" s="2" t="inlineStr"/>
+      <c r="T60" s="2" t="inlineStr">
+        <is>
+          <t>nces: no match</t>
+        </is>
+      </c>
     </row>
     <row r="61">
       <c r="A61" t="inlineStr">
@@ -7816,7 +7927,11 @@
           <t>https://en.wikipedia.org/wiki/Rose_Parade_marching_bands</t>
         </is>
       </c>
-      <c r="T61" s="2" t="inlineStr"/>
+      <c r="T61" s="2" t="inlineStr">
+        <is>
+          <t>nces: no match</t>
+        </is>
+      </c>
     </row>
     <row r="62">
       <c r="A62" t="inlineStr">
@@ -7868,7 +7983,11 @@
           <t>https://en.wikipedia.org/wiki/Rose_Parade_marching_bands</t>
         </is>
       </c>
-      <c r="T62" s="2" t="inlineStr"/>
+      <c r="T62" s="2" t="inlineStr">
+        <is>
+          <t>nces: no match</t>
+        </is>
+      </c>
     </row>
     <row r="63">
       <c r="A63" t="inlineStr">
@@ -7911,20 +8030,43 @@
         <v>2018</v>
       </c>
       <c r="J63" t="inlineStr"/>
-      <c r="K63" t="inlineStr"/>
-      <c r="L63" t="inlineStr"/>
-      <c r="M63" t="inlineStr"/>
-      <c r="N63" t="inlineStr"/>
+      <c r="K63" t="inlineStr">
+        <is>
+          <t>MANATEE</t>
+        </is>
+      </c>
+      <c r="L63" t="n">
+        <v>1801</v>
+      </c>
+      <c r="M63" t="inlineStr">
+        <is>
+          <t>http://www.manateeschools.net/bradenriver</t>
+        </is>
+      </c>
+      <c r="N63" t="inlineStr">
+        <is>
+          <t>http://www.manateeschools.net/bradenriver</t>
+        </is>
+      </c>
       <c r="O63" t="inlineStr"/>
       <c r="P63" t="inlineStr"/>
       <c r="Q63" t="inlineStr"/>
-      <c r="R63" t="inlineStr"/>
+      <c r="R63" t="inlineStr">
+        <is>
+          <t>Communications Show submenu for Arts and Communications Band Boosters Pirate Nation News Business a</t>
+        </is>
+      </c>
       <c r="S63" s="2" t="inlineStr">
         <is>
-          <t>https://en.wikipedia.org/wiki/6abc_Dunkin%27_Thanksgiving_Day_Parade</t>
-        </is>
-      </c>
-      <c r="T63" s="2" t="inlineStr"/>
+          <t>https://en.wikipedia.org/wiki/6abc_Dunkin%27_Thanksgiving_Day_Parade
+http://www.manateeschools.net/bradenriver</t>
+        </is>
+      </c>
+      <c r="T63" s="2" t="inlineStr">
+        <is>
+          <t>social: https://www.facebook.com/BRHSPirateNation; social: https://www.facebook.com/BradenRiverHSBands; social: https://www.instagram.com/bradenriverhsbands</t>
+        </is>
+      </c>
     </row>
     <row r="64">
       <c r="A64" t="inlineStr">
@@ -7970,7 +8112,7 @@
       </c>
       <c r="T64" s="2" t="inlineStr">
         <is>
-          <t>state unknown: source lists no location</t>
+          <t>state unknown: source lists no location; nces: skipped (state unknown)</t>
         </is>
       </c>
     </row>
@@ -8015,8 +8157,14 @@
         <v>2018</v>
       </c>
       <c r="J65" t="inlineStr"/>
-      <c r="K65" t="inlineStr"/>
-      <c r="L65" t="inlineStr"/>
+      <c r="K65" t="inlineStr">
+        <is>
+          <t>OKALOOSA</t>
+        </is>
+      </c>
+      <c r="L65" t="n">
+        <v>2397</v>
+      </c>
       <c r="M65" t="inlineStr"/>
       <c r="N65" t="inlineStr"/>
       <c r="O65" t="inlineStr"/>
@@ -8028,7 +8176,11 @@
           <t>https://en.wikipedia.org/wiki/6abc_Dunkin%27_Thanksgiving_Day_Parade</t>
         </is>
       </c>
-      <c r="T65" s="2" t="inlineStr"/>
+      <c r="T65" s="2" t="inlineStr">
+        <is>
+          <t>no website in NCES</t>
+        </is>
+      </c>
     </row>
     <row r="66">
       <c r="A66" t="inlineStr">
@@ -8071,9 +8223,19 @@
         <v>2015</v>
       </c>
       <c r="J66" t="inlineStr"/>
-      <c r="K66" t="inlineStr"/>
-      <c r="L66" t="inlineStr"/>
-      <c r="M66" t="inlineStr"/>
+      <c r="K66" t="inlineStr">
+        <is>
+          <t>Anaheim Union High</t>
+        </is>
+      </c>
+      <c r="L66" t="n">
+        <v>2705</v>
+      </c>
+      <c r="M66" t="inlineStr">
+        <is>
+          <t>http://cypress.auhsd.us</t>
+        </is>
+      </c>
       <c r="N66" t="inlineStr"/>
       <c r="O66" t="inlineStr"/>
       <c r="P66" t="inlineStr"/>
@@ -8084,7 +8246,11 @@
           <t>https://en.wikipedia.org/wiki/Rose_Parade_marching_bands</t>
         </is>
       </c>
-      <c r="T66" s="2" t="inlineStr"/>
+      <c r="T66" s="2" t="inlineStr">
+        <is>
+          <t>nces: matched 'Cypress High' (0.92); no band page found in 3 pages crawled</t>
+        </is>
+      </c>
     </row>
     <row r="67">
       <c r="A67" t="inlineStr">
@@ -8134,7 +8300,7 @@
       </c>
       <c r="T67" s="2" t="inlineStr">
         <is>
-          <t>state unknown: source lists no location</t>
+          <t>state unknown: source lists no location; nces: skipped (state unknown)</t>
         </is>
       </c>
     </row>
@@ -8188,7 +8354,11 @@
           <t>https://en.wikipedia.org/wiki/Rose_Parade_marching_bands</t>
         </is>
       </c>
-      <c r="T68" s="2" t="inlineStr"/>
+      <c r="T68" s="2" t="inlineStr">
+        <is>
+          <t>nces: no match</t>
+        </is>
+      </c>
     </row>
     <row r="69">
       <c r="A69" t="inlineStr">
@@ -8227,8 +8397,14 @@
         <v>2017</v>
       </c>
       <c r="J69" t="inlineStr"/>
-      <c r="K69" t="inlineStr"/>
-      <c r="L69" t="inlineStr"/>
+      <c r="K69" t="inlineStr">
+        <is>
+          <t>Clark County</t>
+        </is>
+      </c>
+      <c r="L69" t="n">
+        <v>2362</v>
+      </c>
       <c r="M69" t="inlineStr"/>
       <c r="N69" t="inlineStr"/>
       <c r="O69" t="inlineStr"/>
@@ -8240,7 +8416,11 @@
           <t>https://en.wikipedia.org/wiki/Rose_Parade_marching_bands</t>
         </is>
       </c>
-      <c r="T69" s="2" t="inlineStr"/>
+      <c r="T69" s="2" t="inlineStr">
+        <is>
+          <t>no website in NCES</t>
+        </is>
+      </c>
     </row>
     <row r="70">
       <c r="A70" t="inlineStr">
@@ -8283,9 +8463,19 @@
         <v>2016</v>
       </c>
       <c r="J70" t="inlineStr"/>
-      <c r="K70" t="inlineStr"/>
-      <c r="L70" t="inlineStr"/>
-      <c r="M70" t="inlineStr"/>
+      <c r="K70" t="inlineStr">
+        <is>
+          <t>Franklin Regional SD</t>
+        </is>
+      </c>
+      <c r="L70" t="n">
+        <v>1106</v>
+      </c>
+      <c r="M70" t="inlineStr">
+        <is>
+          <t>http://highschool.frsdk12.org/</t>
+        </is>
+      </c>
       <c r="N70" t="inlineStr"/>
       <c r="O70" t="inlineStr"/>
       <c r="P70" t="inlineStr"/>
@@ -8296,7 +8486,11 @@
           <t>https://en.wikipedia.org/wiki/Rose_Parade_marching_bands</t>
         </is>
       </c>
-      <c r="T70" s="2" t="inlineStr"/>
+      <c r="T70" s="2" t="inlineStr">
+        <is>
+          <t>nces: matched 'Franklin Regional SHS' (0.92); no band page found in 1 pages crawled</t>
+        </is>
+      </c>
     </row>
     <row r="71">
       <c r="A71" t="inlineStr">
@@ -8335,8 +8529,14 @@
         <v>2017</v>
       </c>
       <c r="J71" t="inlineStr"/>
-      <c r="K71" t="inlineStr"/>
-      <c r="L71" t="inlineStr"/>
+      <c r="K71" t="inlineStr">
+        <is>
+          <t>South-Western City</t>
+        </is>
+      </c>
+      <c r="L71" t="n">
+        <v>1853</v>
+      </c>
       <c r="M71" t="inlineStr"/>
       <c r="N71" t="inlineStr"/>
       <c r="O71" t="inlineStr"/>
@@ -8348,7 +8548,11 @@
           <t>https://en.wikipedia.org/wiki/Rose_Parade_marching_bands</t>
         </is>
       </c>
-      <c r="T71" s="2" t="inlineStr"/>
+      <c r="T71" s="2" t="inlineStr">
+        <is>
+          <t>no website in NCES</t>
+        </is>
+      </c>
     </row>
     <row r="72">
       <c r="A72" t="inlineStr">
@@ -8391,9 +8595,19 @@
         <v>2019</v>
       </c>
       <c r="J72" t="inlineStr"/>
-      <c r="K72" t="inlineStr"/>
-      <c r="L72" t="inlineStr"/>
-      <c r="M72" t="inlineStr"/>
+      <c r="K72" t="inlineStr">
+        <is>
+          <t>COLLIER</t>
+        </is>
+      </c>
+      <c r="L72" t="n">
+        <v>1831</v>
+      </c>
+      <c r="M72" t="inlineStr">
+        <is>
+          <t>http://www.collierschools.com/gch</t>
+        </is>
+      </c>
       <c r="N72" t="inlineStr"/>
       <c r="O72" t="inlineStr"/>
       <c r="P72" t="inlineStr"/>
@@ -8404,7 +8618,11 @@
           <t>https://en.wikipedia.org/wiki/6abc_Dunkin%27_Thanksgiving_Day_Parade</t>
         </is>
       </c>
-      <c r="T72" s="2" t="inlineStr"/>
+      <c r="T72" s="2" t="inlineStr">
+        <is>
+          <t>no band page found in 1 pages crawled</t>
+        </is>
+      </c>
     </row>
     <row r="73">
       <c r="A73" t="inlineStr">
@@ -8454,7 +8672,7 @@
       </c>
       <c r="T73" s="2" t="inlineStr">
         <is>
-          <t>state unknown: source lists no location</t>
+          <t>state unknown: source lists no location; nces: skipped (state unknown)</t>
         </is>
       </c>
     </row>
@@ -8499,9 +8717,19 @@
         <v>2019</v>
       </c>
       <c r="J74" t="inlineStr"/>
-      <c r="K74" t="inlineStr"/>
-      <c r="L74" t="inlineStr"/>
-      <c r="M74" t="inlineStr"/>
+      <c r="K74" t="inlineStr">
+        <is>
+          <t>Fontana Unified</t>
+        </is>
+      </c>
+      <c r="L74" t="n">
+        <v>1794</v>
+      </c>
+      <c r="M74" t="inlineStr">
+        <is>
+          <t>http://www.fusd.net</t>
+        </is>
+      </c>
       <c r="N74" t="inlineStr"/>
       <c r="O74" t="inlineStr"/>
       <c r="P74" t="inlineStr"/>
@@ -8512,7 +8740,11 @@
           <t>https://en.wikipedia.org/wiki/Rose_Parade_marching_bands</t>
         </is>
       </c>
-      <c r="T74" s="2" t="inlineStr"/>
+      <c r="T74" s="2" t="inlineStr">
+        <is>
+          <t>nces: matched 'Henry J. Kaiser High' (0.92); no band page found in 11 pages crawled</t>
+        </is>
+      </c>
     </row>
     <row r="75">
       <c r="A75" t="inlineStr">
@@ -8564,7 +8796,11 @@
           <t>https://en.wikipedia.org/wiki/Rose_Parade_marching_bands</t>
         </is>
       </c>
-      <c r="T75" s="2" t="inlineStr"/>
+      <c r="T75" s="2" t="inlineStr">
+        <is>
+          <t>nces: no match</t>
+        </is>
+      </c>
     </row>
     <row r="76">
       <c r="A76" t="inlineStr">
@@ -8607,8 +8843,14 @@
         <v>2015</v>
       </c>
       <c r="J76" t="inlineStr"/>
-      <c r="K76" t="inlineStr"/>
-      <c r="L76" t="inlineStr"/>
+      <c r="K76" t="inlineStr">
+        <is>
+          <t>Lakota Local</t>
+        </is>
+      </c>
+      <c r="L76" t="n">
+        <v>2845</v>
+      </c>
       <c r="M76" t="inlineStr"/>
       <c r="N76" t="inlineStr"/>
       <c r="O76" t="inlineStr"/>
@@ -8620,7 +8862,11 @@
           <t>https://en.wikipedia.org/wiki/Rose_Parade_marching_bands</t>
         </is>
       </c>
-      <c r="T76" s="2" t="inlineStr"/>
+      <c r="T76" s="2" t="inlineStr">
+        <is>
+          <t>no website in NCES</t>
+        </is>
+      </c>
     </row>
     <row r="77">
       <c r="A77" t="inlineStr">
@@ -8663,8 +8909,14 @@
         <v>2015</v>
       </c>
       <c r="J77" t="inlineStr"/>
-      <c r="K77" t="inlineStr"/>
-      <c r="L77" t="inlineStr"/>
+      <c r="K77" t="inlineStr">
+        <is>
+          <t>Adams 12 Five Star Schools</t>
+        </is>
+      </c>
+      <c r="L77" t="n">
+        <v>2158</v>
+      </c>
       <c r="M77" t="inlineStr"/>
       <c r="N77" t="inlineStr"/>
       <c r="O77" t="inlineStr"/>
@@ -8676,7 +8928,11 @@
           <t>https://en.wikipedia.org/wiki/Rose_Parade_marching_bands</t>
         </is>
       </c>
-      <c r="T77" s="2" t="inlineStr"/>
+      <c r="T77" s="2" t="inlineStr">
+        <is>
+          <t>no website in NCES</t>
+        </is>
+      </c>
     </row>
     <row r="78">
       <c r="A78" t="inlineStr">
@@ -8726,7 +8982,7 @@
       </c>
       <c r="T78" s="2" t="inlineStr">
         <is>
-          <t>state unknown: source lists no location</t>
+          <t>state unknown: source lists no location; nces: skipped (state unknown)</t>
         </is>
       </c>
     </row>
@@ -8771,9 +9027,19 @@
         <v>2018</v>
       </c>
       <c r="J79" t="inlineStr"/>
-      <c r="K79" t="inlineStr"/>
-      <c r="L79" t="inlineStr"/>
-      <c r="M79" t="inlineStr"/>
+      <c r="K79" t="inlineStr">
+        <is>
+          <t>LINDBERGH SCHOOLS</t>
+        </is>
+      </c>
+      <c r="L79" t="n">
+        <v>2266</v>
+      </c>
+      <c r="M79" t="inlineStr">
+        <is>
+          <t>http://go.lindberghschools.ws/Domain/8</t>
+        </is>
+      </c>
       <c r="N79" t="inlineStr"/>
       <c r="O79" t="inlineStr"/>
       <c r="P79" t="inlineStr"/>
@@ -8784,7 +9050,11 @@
           <t>https://en.wikipedia.org/wiki/Rose_Parade_marching_bands</t>
         </is>
       </c>
-      <c r="T79" s="2" t="inlineStr"/>
+      <c r="T79" s="2" t="inlineStr">
+        <is>
+          <t>nces: matched 'LINDBERGH SR. HIGH' (0.92); site crawl blocked: HTTP 404 for http://go.lindberghschools.ws/Domain/8</t>
+        </is>
+      </c>
     </row>
     <row r="80">
       <c r="A80" t="inlineStr">
@@ -8827,9 +9097,19 @@
         <v>2018</v>
       </c>
       <c r="J80" t="inlineStr"/>
-      <c r="K80" t="inlineStr"/>
-      <c r="L80" t="inlineStr"/>
-      <c r="M80" t="inlineStr"/>
+      <c r="K80" t="inlineStr">
+        <is>
+          <t>Londonderry School District</t>
+        </is>
+      </c>
+      <c r="L80" t="n">
+        <v>1308</v>
+      </c>
+      <c r="M80" t="inlineStr">
+        <is>
+          <t>http://www.londonderry.org/lhs</t>
+        </is>
+      </c>
       <c r="N80" t="inlineStr"/>
       <c r="O80" t="inlineStr"/>
       <c r="P80" t="inlineStr"/>
@@ -8840,7 +9120,11 @@
           <t>https://en.wikipedia.org/wiki/Rose_Parade_marching_bands</t>
         </is>
       </c>
-      <c r="T80" s="2" t="inlineStr"/>
+      <c r="T80" s="2" t="inlineStr">
+        <is>
+          <t>site crawl blocked: HTTP 404 for http://www.londonderry.org/lhs</t>
+        </is>
+      </c>
     </row>
     <row r="81">
       <c r="A81" t="inlineStr">
@@ -8883,9 +9167,19 @@
         <v>2018</v>
       </c>
       <c r="J81" t="inlineStr"/>
-      <c r="K81" t="inlineStr"/>
-      <c r="L81" t="inlineStr"/>
-      <c r="M81" t="inlineStr"/>
+      <c r="K81" t="inlineStr">
+        <is>
+          <t>Louisburg</t>
+        </is>
+      </c>
+      <c r="L81" t="n">
+        <v>540</v>
+      </c>
+      <c r="M81" t="inlineStr">
+        <is>
+          <t>http://www.usd416.org</t>
+        </is>
+      </c>
       <c r="N81" t="inlineStr"/>
       <c r="O81" t="inlineStr"/>
       <c r="P81" t="inlineStr"/>
@@ -8896,7 +9190,11 @@
           <t>https://en.wikipedia.org/wiki/Rose_Parade_marching_bands</t>
         </is>
       </c>
-      <c r="T81" s="2" t="inlineStr"/>
+      <c r="T81" s="2" t="inlineStr">
+        <is>
+          <t>nces: matched 'Louisburg High' (0.92); no band page found in 1 pages crawled</t>
+        </is>
+      </c>
     </row>
     <row r="82">
       <c r="A82" t="inlineStr">
@@ -8942,7 +9240,7 @@
       </c>
       <c r="T82" s="2" t="inlineStr">
         <is>
-          <t>state unknown: source lists no location</t>
+          <t>state unknown: source lists no location; nces: skipped (state unknown)</t>
         </is>
       </c>
     </row>
@@ -8996,7 +9294,11 @@
           <t>https://en.wikipedia.org/wiki/Rose_Parade_marching_bands</t>
         </is>
       </c>
-      <c r="T83" s="2" t="inlineStr"/>
+      <c r="T83" s="2" t="inlineStr">
+        <is>
+          <t>nces: no match</t>
+        </is>
+      </c>
     </row>
     <row r="84">
       <c r="A84" t="inlineStr">
@@ -9039,8 +9341,14 @@
         <v>2015</v>
       </c>
       <c r="J84" t="inlineStr"/>
-      <c r="K84" t="inlineStr"/>
-      <c r="L84" t="inlineStr"/>
+      <c r="K84" t="inlineStr">
+        <is>
+          <t>Hawaii Department of Education</t>
+        </is>
+      </c>
+      <c r="L84" t="n">
+        <v>1908</v>
+      </c>
       <c r="M84" t="inlineStr"/>
       <c r="N84" t="inlineStr"/>
       <c r="O84" t="inlineStr"/>
@@ -9052,7 +9360,11 @@
           <t>https://en.wikipedia.org/wiki/Rose_Parade_marching_bands</t>
         </is>
       </c>
-      <c r="T84" s="2" t="inlineStr"/>
+      <c r="T84" s="2" t="inlineStr">
+        <is>
+          <t>no website in NCES</t>
+        </is>
+      </c>
     </row>
     <row r="85">
       <c r="A85" t="inlineStr">
@@ -9095,8 +9407,14 @@
         <v>2019</v>
       </c>
       <c r="J85" t="inlineStr"/>
-      <c r="K85" t="inlineStr"/>
-      <c r="L85" t="inlineStr"/>
+      <c r="K85" t="inlineStr">
+        <is>
+          <t>Mercer Island School District</t>
+        </is>
+      </c>
+      <c r="L85" t="n">
+        <v>1465</v>
+      </c>
       <c r="M85" t="inlineStr"/>
       <c r="N85" t="inlineStr"/>
       <c r="O85" t="inlineStr"/>
@@ -9108,7 +9426,11 @@
           <t>https://en.wikipedia.org/wiki/Rose_Parade_marching_bands</t>
         </is>
       </c>
-      <c r="T85" s="2" t="inlineStr"/>
+      <c r="T85" s="2" t="inlineStr">
+        <is>
+          <t>no website in NCES</t>
+        </is>
+      </c>
     </row>
     <row r="86">
       <c r="A86" t="inlineStr">
@@ -9158,7 +9480,7 @@
       </c>
       <c r="T86" s="2" t="inlineStr">
         <is>
-          <t>state unknown: source lists no location</t>
+          <t>state unknown: source lists no location; nces: skipped (state unknown)</t>
         </is>
       </c>
     </row>
@@ -9210,7 +9532,7 @@
       </c>
       <c r="T87" s="2" t="inlineStr">
         <is>
-          <t>state unknown: source lists no location</t>
+          <t>state unknown: source lists no location; nces: skipped (state unknown)</t>
         </is>
       </c>
     </row>
@@ -9262,7 +9584,7 @@
       </c>
       <c r="T88" s="2" t="inlineStr">
         <is>
-          <t>state unknown: source lists no location</t>
+          <t>state unknown: source lists no location; nces: skipped (state unknown)</t>
         </is>
       </c>
     </row>
@@ -9320,7 +9642,11 @@
           <t>https://en.wikipedia.org/wiki/Rose_Parade_marching_bands</t>
         </is>
       </c>
-      <c r="T89" s="2" t="inlineStr"/>
+      <c r="T89" s="2" t="inlineStr">
+        <is>
+          <t>nces: no match</t>
+        </is>
+      </c>
     </row>
     <row r="90">
       <c r="A90" t="inlineStr">
@@ -9372,7 +9698,11 @@
           <t>https://en.wikipedia.org/wiki/Rose_Parade_marching_bands</t>
         </is>
       </c>
-      <c r="T90" s="2" t="inlineStr"/>
+      <c r="T90" s="2" t="inlineStr">
+        <is>
+          <t>nces: no match</t>
+        </is>
+      </c>
     </row>
     <row r="91">
       <c r="A91" t="inlineStr">
@@ -9422,7 +9752,7 @@
       </c>
       <c r="T91" s="2" t="inlineStr">
         <is>
-          <t>state unknown: source lists no location</t>
+          <t>state unknown: source lists no location; nces: skipped (state unknown)</t>
         </is>
       </c>
     </row>
@@ -9480,7 +9810,11 @@
           <t>https://en.wikipedia.org/wiki/Rose_Parade_marching_bands</t>
         </is>
       </c>
-      <c r="T92" s="2" t="inlineStr"/>
+      <c r="T92" s="2" t="inlineStr">
+        <is>
+          <t>nces: no match</t>
+        </is>
+      </c>
     </row>
     <row r="93">
       <c r="A93" t="inlineStr">
@@ -9579,20 +9913,39 @@
         <v>2016</v>
       </c>
       <c r="J94" t="inlineStr"/>
-      <c r="K94" t="inlineStr"/>
-      <c r="L94" t="inlineStr"/>
-      <c r="M94" t="inlineStr"/>
-      <c r="N94" t="inlineStr"/>
+      <c r="K94" t="inlineStr">
+        <is>
+          <t>Los Gatos-Saratoga Union High</t>
+        </is>
+      </c>
+      <c r="L94" t="n">
+        <v>1198</v>
+      </c>
+      <c r="M94" t="inlineStr">
+        <is>
+          <t>http://www.saratogahigh.org</t>
+        </is>
+      </c>
+      <c r="N94" t="inlineStr">
+        <is>
+          <t>https://www.saratogamusicboosters.org/</t>
+        </is>
+      </c>
       <c r="O94" t="inlineStr"/>
       <c r="P94" t="inlineStr"/>
       <c r="Q94" t="inlineStr"/>
       <c r="R94" t="inlineStr"/>
       <c r="S94" s="2" t="inlineStr">
         <is>
-          <t>https://en.wikipedia.org/wiki/Rose_Parade_marching_bands</t>
-        </is>
-      </c>
-      <c r="T94" s="2" t="inlineStr"/>
+          <t>https://en.wikipedia.org/wiki/Rose_Parade_marching_bands
+https://www.saratogamusicboosters.org/</t>
+        </is>
+      </c>
+      <c r="T94" s="2" t="inlineStr">
+        <is>
+          <t>nces: matched 'Saratoga High' (0.92); social: https://www.instagram.com/saratogamusicboosters; social: https://www.facebook.com/saratogamusicboosters; social: https://www.instagram.com/reel/CxUE6_IpT2c</t>
+        </is>
+      </c>
     </row>
     <row r="95">
       <c r="A95" t="inlineStr">
@@ -9638,7 +9991,7 @@
       </c>
       <c r="T95" s="2" t="inlineStr">
         <is>
-          <t>state unknown: source lists no location</t>
+          <t>state unknown: source lists no location; nces: skipped (state unknown)</t>
         </is>
       </c>
     </row>
@@ -9683,8 +10036,14 @@
         <v>2015</v>
       </c>
       <c r="J96" t="inlineStr"/>
-      <c r="K96" t="inlineStr"/>
-      <c r="L96" t="inlineStr"/>
+      <c r="K96" t="inlineStr">
+        <is>
+          <t>Temple City Unified</t>
+        </is>
+      </c>
+      <c r="L96" t="n">
+        <v>1758</v>
+      </c>
       <c r="M96" t="inlineStr"/>
       <c r="N96" t="inlineStr"/>
       <c r="O96" t="inlineStr"/>
@@ -9696,7 +10055,11 @@
           <t>https://en.wikipedia.org/wiki/Rose_Parade_marching_bands</t>
         </is>
       </c>
-      <c r="T96" s="2" t="inlineStr"/>
+      <c r="T96" s="2" t="inlineStr">
+        <is>
+          <t>nces: matched 'Temple City High' (0.92); no website in NCES</t>
+        </is>
+      </c>
     </row>
     <row r="97">
       <c r="A97" t="inlineStr">
@@ -9748,7 +10111,11 @@
           <t>https://en.wikipedia.org/wiki/Rose_Parade_marching_bands</t>
         </is>
       </c>
-      <c r="T97" s="2" t="inlineStr"/>
+      <c r="T97" s="2" t="inlineStr">
+        <is>
+          <t>nces: no match</t>
+        </is>
+      </c>
     </row>
     <row r="98">
       <c r="A98" t="inlineStr">
@@ -9791,9 +10158,19 @@
         <v>2018</v>
       </c>
       <c r="J98" t="inlineStr"/>
-      <c r="K98" t="inlineStr"/>
-      <c r="L98" t="inlineStr"/>
-      <c r="M98" t="inlineStr"/>
+      <c r="K98" t="inlineStr">
+        <is>
+          <t>Alpine District</t>
+        </is>
+      </c>
+      <c r="L98" t="n">
+        <v>2847</v>
+      </c>
+      <c r="M98" t="inlineStr">
+        <is>
+          <t>http://westlake.alpinedistrict.org/</t>
+        </is>
+      </c>
       <c r="N98" t="inlineStr"/>
       <c r="O98" t="inlineStr"/>
       <c r="P98" t="inlineStr"/>
@@ -9804,7 +10181,11 @@
           <t>https://en.wikipedia.org/wiki/Rose_Parade_marching_bands</t>
         </is>
       </c>
-      <c r="T98" s="2" t="inlineStr"/>
+      <c r="T98" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">nces: matched 'Westlake High' (0.92); site crawl blocked: TLS failure for http://westlake.alpinedistrict.org/: HTTPSConnectionPool(host='westlake.alpinedistrict.org', port=443): </t>
+        </is>
+      </c>
     </row>
     <row r="99">
       <c r="A99" t="inlineStr">
@@ -9909,9 +10290,19 @@
         <v>2019</v>
       </c>
       <c r="J100" t="inlineStr"/>
-      <c r="K100" t="inlineStr"/>
-      <c r="L100" t="inlineStr"/>
-      <c r="M100" t="inlineStr"/>
+      <c r="K100" t="inlineStr">
+        <is>
+          <t>Decatur County</t>
+        </is>
+      </c>
+      <c r="L100" t="n">
+        <v>1218</v>
+      </c>
+      <c r="M100" t="inlineStr">
+        <is>
+          <t>http://bhs.boe.dcboe.com/</t>
+        </is>
+      </c>
       <c r="N100" t="inlineStr"/>
       <c r="O100" t="inlineStr"/>
       <c r="P100" t="inlineStr"/>
@@ -9922,7 +10313,11 @@
           <t>https://en.wikipedia.org/wiki/6abc_Dunkin%27_Thanksgiving_Day_Parade</t>
         </is>
       </c>
-      <c r="T100" s="2" t="inlineStr"/>
+      <c r="T100" s="2" t="inlineStr">
+        <is>
+          <t>no band page found in 1 pages crawled</t>
+        </is>
+      </c>
     </row>
     <row r="101">
       <c r="A101" t="inlineStr">
@@ -9965,9 +10360,19 @@
         <v>2016</v>
       </c>
       <c r="J101" t="inlineStr"/>
-      <c r="K101" t="inlineStr"/>
-      <c r="L101" t="inlineStr"/>
-      <c r="M101" t="inlineStr"/>
+      <c r="K101" t="inlineStr">
+        <is>
+          <t>Lauderdale County</t>
+        </is>
+      </c>
+      <c r="L101" t="n">
+        <v>744</v>
+      </c>
+      <c r="M101" t="inlineStr">
+        <is>
+          <t>http://www.lcschools.org</t>
+        </is>
+      </c>
       <c r="N101" t="inlineStr"/>
       <c r="O101" t="inlineStr"/>
       <c r="P101" t="inlineStr"/>
@@ -9978,7 +10383,11 @@
           <t>https://en.wikipedia.org/wiki/6abc_Dunkin%27_Thanksgiving_Day_Parade</t>
         </is>
       </c>
-      <c r="T101" s="2" t="inlineStr"/>
+      <c r="T101" s="2" t="inlineStr">
+        <is>
+          <t>no band page found in 1 pages crawled</t>
+        </is>
+      </c>
     </row>
   </sheetData>
   <autoFilter ref="A1:T101"/>
@@ -10300,12 +10709,12 @@
       </c>
       <c r="D4" t="inlineStr">
         <is>
-          <t>The Pride of</t>
+          <t>The Pride of Broken Arrow</t>
         </is>
       </c>
       <c r="E4" t="inlineStr">
         <is>
-          <t>The Pride of Broken Arrow</t>
+          <t>Broken Arrow</t>
         </is>
       </c>
       <c r="F4" t="inlineStr">
@@ -12752,7 +13161,7 @@
       </c>
       <c r="E38" t="inlineStr">
         <is>
-          <t>Red Raider Marching Band</t>
+          <t>Pulaski</t>
         </is>
       </c>
       <c r="F38" t="inlineStr">
@@ -15744,20 +16153,43 @@
         <v>2019</v>
       </c>
       <c r="J86" t="inlineStr"/>
-      <c r="K86" t="inlineStr"/>
-      <c r="L86" t="inlineStr"/>
-      <c r="M86" t="inlineStr"/>
-      <c r="N86" t="inlineStr"/>
+      <c r="K86" t="inlineStr">
+        <is>
+          <t>Cobb County</t>
+        </is>
+      </c>
+      <c r="L86" t="n">
+        <v>1949</v>
+      </c>
+      <c r="M86" t="inlineStr">
+        <is>
+          <t>http://www.cobbk12.org/lassiter</t>
+        </is>
+      </c>
+      <c r="N86" t="inlineStr">
+        <is>
+          <t>http://www.cobbk12.org/lassiter/band</t>
+        </is>
+      </c>
       <c r="O86" t="inlineStr"/>
       <c r="P86" t="inlineStr"/>
       <c r="Q86" t="inlineStr"/>
-      <c r="R86" t="inlineStr"/>
+      <c r="R86" t="inlineStr">
+        <is>
+          <t>Our supportive parent community and Lassiter Band Booster Association raise funds that</t>
+        </is>
+      </c>
       <c r="S86" s="2" t="inlineStr">
         <is>
-          <t>https://en.wikipedia.org/wiki/Rose_Parade_marching_bands</t>
-        </is>
-      </c>
-      <c r="T86" s="2" t="inlineStr"/>
+          <t>https://en.wikipedia.org/wiki/Rose_Parade_marching_bands
+http://www.cobbk12.org/lassiter/band</t>
+        </is>
+      </c>
+      <c r="T86" s="2" t="inlineStr">
+        <is>
+          <t>social: https://www.facebook.com/cobbschools</t>
+        </is>
+      </c>
     </row>
     <row r="87">
       <c r="A87" t="inlineStr">
@@ -15876,9 +16308,19 @@
         <v>2019</v>
       </c>
       <c r="J88" t="inlineStr"/>
-      <c r="K88" t="inlineStr"/>
-      <c r="L88" t="inlineStr"/>
-      <c r="M88" t="inlineStr"/>
+      <c r="K88" t="inlineStr">
+        <is>
+          <t>Tipton County</t>
+        </is>
+      </c>
+      <c r="L88" t="n">
+        <v>1273</v>
+      </c>
+      <c r="M88" t="inlineStr">
+        <is>
+          <t>http://www.tipton-county.com/mhs</t>
+        </is>
+      </c>
       <c r="N88" t="inlineStr"/>
       <c r="O88" t="inlineStr"/>
       <c r="P88" t="inlineStr"/>
@@ -15889,7 +16331,11 @@
           <t>https://en.wikipedia.org/wiki/Rose_Parade_marching_bands</t>
         </is>
       </c>
-      <c r="T88" s="2" t="inlineStr"/>
+      <c r="T88" s="2" t="inlineStr">
+        <is>
+          <t>site crawl blocked: HTTP 403 / challenge page for http://www.tipton-county.com/mhs</t>
+        </is>
+      </c>
     </row>
     <row r="89">
       <c r="A89" t="inlineStr">
@@ -15976,9 +16422,19 @@
         <v>2017</v>
       </c>
       <c r="J90" t="inlineStr"/>
-      <c r="K90" t="inlineStr"/>
-      <c r="L90" t="inlineStr"/>
-      <c r="M90" t="inlineStr"/>
+      <c r="K90" t="inlineStr">
+        <is>
+          <t>Hamilton County</t>
+        </is>
+      </c>
+      <c r="L90" t="n">
+        <v>1275</v>
+      </c>
+      <c r="M90" t="inlineStr">
+        <is>
+          <t>http://ohs.hcde.org/</t>
+        </is>
+      </c>
       <c r="N90" t="inlineStr"/>
       <c r="O90" t="inlineStr"/>
       <c r="P90" t="inlineStr"/>
@@ -15989,7 +16445,11 @@
           <t>https://en.wikipedia.org/wiki/Rose_Parade_marching_bands</t>
         </is>
       </c>
-      <c r="T90" s="2" t="inlineStr"/>
+      <c r="T90" s="2" t="inlineStr">
+        <is>
+          <t>no band page found in 2 pages crawled</t>
+        </is>
+      </c>
     </row>
     <row r="91">
       <c r="A91" t="inlineStr">
@@ -16366,9 +16826,19 @@
         <v>2015</v>
       </c>
       <c r="J96" t="inlineStr"/>
-      <c r="K96" t="inlineStr"/>
-      <c r="L96" t="inlineStr"/>
-      <c r="M96" t="inlineStr"/>
+      <c r="K96" t="inlineStr">
+        <is>
+          <t>Cobb County</t>
+        </is>
+      </c>
+      <c r="L96" t="n">
+        <v>2685</v>
+      </c>
+      <c r="M96" t="inlineStr">
+        <is>
+          <t>http://www.waltonhigh.org</t>
+        </is>
+      </c>
       <c r="N96" t="inlineStr"/>
       <c r="O96" t="inlineStr"/>
       <c r="P96" t="inlineStr"/>
@@ -16379,7 +16849,11 @@
           <t>https://en.wikipedia.org/wiki/Rose_Parade_marching_bands</t>
         </is>
       </c>
-      <c r="T96" s="2" t="inlineStr"/>
+      <c r="T96" s="2" t="inlineStr">
+        <is>
+          <t>no band page found in 1 pages crawled</t>
+        </is>
+      </c>
     </row>
     <row r="97">
       <c r="A97" t="inlineStr">
@@ -16577,7 +17051,7 @@
       </c>
       <c r="T99" s="2" t="inlineStr">
         <is>
-          <t>state unknown: source lists no location</t>
+          <t>state unknown: source lists no location; nces: skipped (state unknown)</t>
         </is>
       </c>
     </row>
@@ -16629,7 +17103,7 @@
       </c>
       <c r="T100" s="2" t="inlineStr">
         <is>
-          <t>state unknown: source lists no location</t>
+          <t>state unknown: source lists no location; nces: skipped (state unknown)</t>
         </is>
       </c>
     </row>
@@ -16743,7 +17217,11 @@
           <t>https://en.wikipedia.org/wiki/Rose_Parade_marching_bands</t>
         </is>
       </c>
-      <c r="T102" s="2" t="inlineStr"/>
+      <c r="T102" s="2" t="inlineStr">
+        <is>
+          <t>nces: no match</t>
+        </is>
+      </c>
     </row>
     <row r="103">
       <c r="A103" t="inlineStr">
@@ -16851,7 +17329,11 @@
           <t>https://en.wikipedia.org/wiki/Rose_Parade_marching_bands</t>
         </is>
       </c>
-      <c r="T104" s="2" t="inlineStr"/>
+      <c r="T104" s="2" t="inlineStr">
+        <is>
+          <t>nces: no match</t>
+        </is>
+      </c>
     </row>
     <row r="105">
       <c r="A105" t="inlineStr">
@@ -16894,9 +17376,19 @@
         <v>2020</v>
       </c>
       <c r="J105" t="inlineStr"/>
-      <c r="K105" t="inlineStr"/>
-      <c r="L105" t="inlineStr"/>
-      <c r="M105" t="inlineStr"/>
+      <c r="K105" t="inlineStr">
+        <is>
+          <t>HARRISON CO SCHOOL DIST</t>
+        </is>
+      </c>
+      <c r="L105" t="n">
+        <v>1154</v>
+      </c>
+      <c r="M105" t="inlineStr">
+        <is>
+          <t>http://www.harrison.k12.ms.us/home/westharrisonhigh.aspx</t>
+        </is>
+      </c>
       <c r="N105" t="inlineStr"/>
       <c r="O105" t="inlineStr"/>
       <c r="P105" t="inlineStr"/>
@@ -16907,7 +17399,11 @@
           <t>https://en.wikipedia.org/wiki/Rose_Parade_marching_bands</t>
         </is>
       </c>
-      <c r="T105" s="2" t="inlineStr"/>
+      <c r="T105" s="2" t="inlineStr">
+        <is>
+          <t>no band page found in 1 pages crawled</t>
+        </is>
+      </c>
     </row>
     <row r="106">
       <c r="A106" t="inlineStr">
@@ -16946,8 +17442,14 @@
         <v>2017</v>
       </c>
       <c r="J106" t="inlineStr"/>
-      <c r="K106" t="inlineStr"/>
-      <c r="L106" t="inlineStr"/>
+      <c r="K106" t="inlineStr">
+        <is>
+          <t>EANES ISD</t>
+        </is>
+      </c>
+      <c r="L106" t="n">
+        <v>2811</v>
+      </c>
       <c r="M106" t="inlineStr"/>
       <c r="N106" t="inlineStr"/>
       <c r="O106" t="inlineStr"/>
@@ -16959,7 +17461,11 @@
           <t>https://en.wikipedia.org/wiki/Rose_Parade_marching_bands</t>
         </is>
       </c>
-      <c r="T106" s="2" t="inlineStr"/>
+      <c r="T106" s="2" t="inlineStr">
+        <is>
+          <t>no website in NCES</t>
+        </is>
+      </c>
     </row>
     <row r="107">
       <c r="A107" t="inlineStr">
@@ -17073,7 +17579,7 @@
       </c>
       <c r="T108" s="2" t="inlineStr">
         <is>
-          <t>state unknown: source lists no location</t>
+          <t>state unknown: source lists no location; nces: skipped (state unknown)</t>
         </is>
       </c>
     </row>
@@ -17118,8 +17624,14 @@
         <v>2018</v>
       </c>
       <c r="J109" t="inlineStr"/>
-      <c r="K109" t="inlineStr"/>
-      <c r="L109" t="inlineStr"/>
+      <c r="K109" t="inlineStr">
+        <is>
+          <t>Academy School District No. 20 in the county of El Paso an</t>
+        </is>
+      </c>
+      <c r="L109" t="n">
+        <v>1315</v>
+      </c>
       <c r="M109" t="inlineStr"/>
       <c r="N109" t="inlineStr"/>
       <c r="O109" t="inlineStr"/>
@@ -17131,7 +17643,11 @@
           <t>https://en.wikipedia.org/wiki/Rose_Parade_marching_bands</t>
         </is>
       </c>
-      <c r="T109" s="2" t="inlineStr"/>
+      <c r="T109" s="2" t="inlineStr">
+        <is>
+          <t>no website in NCES</t>
+        </is>
+      </c>
     </row>
     <row r="110">
       <c r="A110" t="inlineStr">
@@ -17187,7 +17703,11 @@
           <t>https://en.wikipedia.org/wiki/Rose_Parade_marching_bands</t>
         </is>
       </c>
-      <c r="T110" s="2" t="inlineStr"/>
+      <c r="T110" s="2" t="inlineStr">
+        <is>
+          <t>nces: no match</t>
+        </is>
+      </c>
     </row>
     <row r="111">
       <c r="A111" t="inlineStr">
@@ -17243,7 +17763,11 @@
           <t>https://en.wikipedia.org/wiki/Rose_Parade_marching_bands</t>
         </is>
       </c>
-      <c r="T111" s="2" t="inlineStr"/>
+      <c r="T111" s="2" t="inlineStr">
+        <is>
+          <t>nces: no match</t>
+        </is>
+      </c>
     </row>
     <row r="112">
       <c r="A112" t="inlineStr">
@@ -17295,7 +17819,11 @@
           <t>https://en.wikipedia.org/wiki/Rose_Parade_marching_bands</t>
         </is>
       </c>
-      <c r="T112" s="2" t="inlineStr"/>
+      <c r="T112" s="2" t="inlineStr">
+        <is>
+          <t>nces: no match</t>
+        </is>
+      </c>
     </row>
     <row r="113">
       <c r="A113" t="inlineStr">
@@ -17338,20 +17866,43 @@
         <v>2018</v>
       </c>
       <c r="J113" t="inlineStr"/>
-      <c r="K113" t="inlineStr"/>
-      <c r="L113" t="inlineStr"/>
-      <c r="M113" t="inlineStr"/>
-      <c r="N113" t="inlineStr"/>
+      <c r="K113" t="inlineStr">
+        <is>
+          <t>MANATEE</t>
+        </is>
+      </c>
+      <c r="L113" t="n">
+        <v>1801</v>
+      </c>
+      <c r="M113" t="inlineStr">
+        <is>
+          <t>http://www.manateeschools.net/bradenriver</t>
+        </is>
+      </c>
+      <c r="N113" t="inlineStr">
+        <is>
+          <t>http://www.manateeschools.net/bradenriver</t>
+        </is>
+      </c>
       <c r="O113" t="inlineStr"/>
       <c r="P113" t="inlineStr"/>
       <c r="Q113" t="inlineStr"/>
-      <c r="R113" t="inlineStr"/>
+      <c r="R113" t="inlineStr">
+        <is>
+          <t>Communications Show submenu for Arts and Communications Band Boosters Pirate Nation News Business a</t>
+        </is>
+      </c>
       <c r="S113" s="2" t="inlineStr">
         <is>
-          <t>https://en.wikipedia.org/wiki/6abc_Dunkin%27_Thanksgiving_Day_Parade</t>
-        </is>
-      </c>
-      <c r="T113" s="2" t="inlineStr"/>
+          <t>https://en.wikipedia.org/wiki/6abc_Dunkin%27_Thanksgiving_Day_Parade
+http://www.manateeschools.net/bradenriver</t>
+        </is>
+      </c>
+      <c r="T113" s="2" t="inlineStr">
+        <is>
+          <t>social: https://www.facebook.com/BRHSPirateNation; social: https://www.facebook.com/BradenRiverHSBands; social: https://www.instagram.com/bradenriverhsbands</t>
+        </is>
+      </c>
     </row>
     <row r="114">
       <c r="A114" t="inlineStr">
@@ -17397,7 +17948,7 @@
       </c>
       <c r="T114" s="2" t="inlineStr">
         <is>
-          <t>state unknown: source lists no location</t>
+          <t>state unknown: source lists no location; nces: skipped (state unknown)</t>
         </is>
       </c>
     </row>
@@ -17442,8 +17993,14 @@
         <v>2018</v>
       </c>
       <c r="J115" t="inlineStr"/>
-      <c r="K115" t="inlineStr"/>
-      <c r="L115" t="inlineStr"/>
+      <c r="K115" t="inlineStr">
+        <is>
+          <t>OKALOOSA</t>
+        </is>
+      </c>
+      <c r="L115" t="n">
+        <v>2397</v>
+      </c>
       <c r="M115" t="inlineStr"/>
       <c r="N115" t="inlineStr"/>
       <c r="O115" t="inlineStr"/>
@@ -17455,7 +18012,11 @@
           <t>https://en.wikipedia.org/wiki/6abc_Dunkin%27_Thanksgiving_Day_Parade</t>
         </is>
       </c>
-      <c r="T115" s="2" t="inlineStr"/>
+      <c r="T115" s="2" t="inlineStr">
+        <is>
+          <t>no website in NCES</t>
+        </is>
+      </c>
     </row>
     <row r="116">
       <c r="A116" t="inlineStr">
@@ -17498,9 +18059,19 @@
         <v>2015</v>
       </c>
       <c r="J116" t="inlineStr"/>
-      <c r="K116" t="inlineStr"/>
-      <c r="L116" t="inlineStr"/>
-      <c r="M116" t="inlineStr"/>
+      <c r="K116" t="inlineStr">
+        <is>
+          <t>Anaheim Union High</t>
+        </is>
+      </c>
+      <c r="L116" t="n">
+        <v>2705</v>
+      </c>
+      <c r="M116" t="inlineStr">
+        <is>
+          <t>http://cypress.auhsd.us</t>
+        </is>
+      </c>
       <c r="N116" t="inlineStr"/>
       <c r="O116" t="inlineStr"/>
       <c r="P116" t="inlineStr"/>
@@ -17511,7 +18082,11 @@
           <t>https://en.wikipedia.org/wiki/Rose_Parade_marching_bands</t>
         </is>
       </c>
-      <c r="T116" s="2" t="inlineStr"/>
+      <c r="T116" s="2" t="inlineStr">
+        <is>
+          <t>nces: matched 'Cypress High' (0.92); no band page found in 3 pages crawled</t>
+        </is>
+      </c>
     </row>
     <row r="117">
       <c r="A117" t="inlineStr">
@@ -17561,7 +18136,7 @@
       </c>
       <c r="T117" s="2" t="inlineStr">
         <is>
-          <t>state unknown: source lists no location</t>
+          <t>state unknown: source lists no location; nces: skipped (state unknown)</t>
         </is>
       </c>
     </row>
@@ -17615,7 +18190,11 @@
           <t>https://en.wikipedia.org/wiki/Rose_Parade_marching_bands</t>
         </is>
       </c>
-      <c r="T118" s="2" t="inlineStr"/>
+      <c r="T118" s="2" t="inlineStr">
+        <is>
+          <t>nces: no match</t>
+        </is>
+      </c>
     </row>
     <row r="119">
       <c r="A119" t="inlineStr">
@@ -17654,8 +18233,14 @@
         <v>2017</v>
       </c>
       <c r="J119" t="inlineStr"/>
-      <c r="K119" t="inlineStr"/>
-      <c r="L119" t="inlineStr"/>
+      <c r="K119" t="inlineStr">
+        <is>
+          <t>Clark County</t>
+        </is>
+      </c>
+      <c r="L119" t="n">
+        <v>2362</v>
+      </c>
       <c r="M119" t="inlineStr"/>
       <c r="N119" t="inlineStr"/>
       <c r="O119" t="inlineStr"/>
@@ -17667,7 +18252,11 @@
           <t>https://en.wikipedia.org/wiki/Rose_Parade_marching_bands</t>
         </is>
       </c>
-      <c r="T119" s="2" t="inlineStr"/>
+      <c r="T119" s="2" t="inlineStr">
+        <is>
+          <t>no website in NCES</t>
+        </is>
+      </c>
     </row>
     <row r="120">
       <c r="A120" t="inlineStr">
@@ -17710,9 +18299,19 @@
         <v>2016</v>
       </c>
       <c r="J120" t="inlineStr"/>
-      <c r="K120" t="inlineStr"/>
-      <c r="L120" t="inlineStr"/>
-      <c r="M120" t="inlineStr"/>
+      <c r="K120" t="inlineStr">
+        <is>
+          <t>Franklin Regional SD</t>
+        </is>
+      </c>
+      <c r="L120" t="n">
+        <v>1106</v>
+      </c>
+      <c r="M120" t="inlineStr">
+        <is>
+          <t>http://highschool.frsdk12.org/</t>
+        </is>
+      </c>
       <c r="N120" t="inlineStr"/>
       <c r="O120" t="inlineStr"/>
       <c r="P120" t="inlineStr"/>
@@ -17723,7 +18322,11 @@
           <t>https://en.wikipedia.org/wiki/Rose_Parade_marching_bands</t>
         </is>
       </c>
-      <c r="T120" s="2" t="inlineStr"/>
+      <c r="T120" s="2" t="inlineStr">
+        <is>
+          <t>nces: matched 'Franklin Regional SHS' (0.92); no band page found in 1 pages crawled</t>
+        </is>
+      </c>
     </row>
     <row r="121">
       <c r="A121" t="inlineStr">
@@ -17762,8 +18365,14 @@
         <v>2017</v>
       </c>
       <c r="J121" t="inlineStr"/>
-      <c r="K121" t="inlineStr"/>
-      <c r="L121" t="inlineStr"/>
+      <c r="K121" t="inlineStr">
+        <is>
+          <t>South-Western City</t>
+        </is>
+      </c>
+      <c r="L121" t="n">
+        <v>1853</v>
+      </c>
       <c r="M121" t="inlineStr"/>
       <c r="N121" t="inlineStr"/>
       <c r="O121" t="inlineStr"/>
@@ -17775,7 +18384,11 @@
           <t>https://en.wikipedia.org/wiki/Rose_Parade_marching_bands</t>
         </is>
       </c>
-      <c r="T121" s="2" t="inlineStr"/>
+      <c r="T121" s="2" t="inlineStr">
+        <is>
+          <t>no website in NCES</t>
+        </is>
+      </c>
     </row>
     <row r="122">
       <c r="A122" t="inlineStr">
@@ -17818,9 +18431,19 @@
         <v>2019</v>
       </c>
       <c r="J122" t="inlineStr"/>
-      <c r="K122" t="inlineStr"/>
-      <c r="L122" t="inlineStr"/>
-      <c r="M122" t="inlineStr"/>
+      <c r="K122" t="inlineStr">
+        <is>
+          <t>COLLIER</t>
+        </is>
+      </c>
+      <c r="L122" t="n">
+        <v>1831</v>
+      </c>
+      <c r="M122" t="inlineStr">
+        <is>
+          <t>http://www.collierschools.com/gch</t>
+        </is>
+      </c>
       <c r="N122" t="inlineStr"/>
       <c r="O122" t="inlineStr"/>
       <c r="P122" t="inlineStr"/>
@@ -17831,7 +18454,11 @@
           <t>https://en.wikipedia.org/wiki/6abc_Dunkin%27_Thanksgiving_Day_Parade</t>
         </is>
       </c>
-      <c r="T122" s="2" t="inlineStr"/>
+      <c r="T122" s="2" t="inlineStr">
+        <is>
+          <t>no band page found in 1 pages crawled</t>
+        </is>
+      </c>
     </row>
     <row r="123">
       <c r="A123" t="inlineStr">
@@ -17881,7 +18508,7 @@
       </c>
       <c r="T123" s="2" t="inlineStr">
         <is>
-          <t>state unknown: source lists no location</t>
+          <t>state unknown: source lists no location; nces: skipped (state unknown)</t>
         </is>
       </c>
     </row>
@@ -17926,9 +18553,19 @@
         <v>2019</v>
       </c>
       <c r="J124" t="inlineStr"/>
-      <c r="K124" t="inlineStr"/>
-      <c r="L124" t="inlineStr"/>
-      <c r="M124" t="inlineStr"/>
+      <c r="K124" t="inlineStr">
+        <is>
+          <t>Fontana Unified</t>
+        </is>
+      </c>
+      <c r="L124" t="n">
+        <v>1794</v>
+      </c>
+      <c r="M124" t="inlineStr">
+        <is>
+          <t>http://www.fusd.net</t>
+        </is>
+      </c>
       <c r="N124" t="inlineStr"/>
       <c r="O124" t="inlineStr"/>
       <c r="P124" t="inlineStr"/>
@@ -17939,7 +18576,11 @@
           <t>https://en.wikipedia.org/wiki/Rose_Parade_marching_bands</t>
         </is>
       </c>
-      <c r="T124" s="2" t="inlineStr"/>
+      <c r="T124" s="2" t="inlineStr">
+        <is>
+          <t>nces: matched 'Henry J. Kaiser High' (0.92); no band page found in 11 pages crawled</t>
+        </is>
+      </c>
     </row>
     <row r="125">
       <c r="A125" t="inlineStr">
@@ -17991,7 +18632,11 @@
           <t>https://en.wikipedia.org/wiki/Rose_Parade_marching_bands</t>
         </is>
       </c>
-      <c r="T125" s="2" t="inlineStr"/>
+      <c r="T125" s="2" t="inlineStr">
+        <is>
+          <t>nces: no match</t>
+        </is>
+      </c>
     </row>
     <row r="126">
       <c r="A126" t="inlineStr">
@@ -18034,8 +18679,14 @@
         <v>2015</v>
       </c>
       <c r="J126" t="inlineStr"/>
-      <c r="K126" t="inlineStr"/>
-      <c r="L126" t="inlineStr"/>
+      <c r="K126" t="inlineStr">
+        <is>
+          <t>Lakota Local</t>
+        </is>
+      </c>
+      <c r="L126" t="n">
+        <v>2845</v>
+      </c>
       <c r="M126" t="inlineStr"/>
       <c r="N126" t="inlineStr"/>
       <c r="O126" t="inlineStr"/>
@@ -18047,7 +18698,11 @@
           <t>https://en.wikipedia.org/wiki/Rose_Parade_marching_bands</t>
         </is>
       </c>
-      <c r="T126" s="2" t="inlineStr"/>
+      <c r="T126" s="2" t="inlineStr">
+        <is>
+          <t>no website in NCES</t>
+        </is>
+      </c>
     </row>
     <row r="127">
       <c r="A127" t="inlineStr">
@@ -18090,8 +18745,14 @@
         <v>2015</v>
       </c>
       <c r="J127" t="inlineStr"/>
-      <c r="K127" t="inlineStr"/>
-      <c r="L127" t="inlineStr"/>
+      <c r="K127" t="inlineStr">
+        <is>
+          <t>Adams 12 Five Star Schools</t>
+        </is>
+      </c>
+      <c r="L127" t="n">
+        <v>2158</v>
+      </c>
       <c r="M127" t="inlineStr"/>
       <c r="N127" t="inlineStr"/>
       <c r="O127" t="inlineStr"/>
@@ -18103,7 +18764,11 @@
           <t>https://en.wikipedia.org/wiki/Rose_Parade_marching_bands</t>
         </is>
       </c>
-      <c r="T127" s="2" t="inlineStr"/>
+      <c r="T127" s="2" t="inlineStr">
+        <is>
+          <t>no website in NCES</t>
+        </is>
+      </c>
     </row>
     <row r="128">
       <c r="A128" t="inlineStr">
@@ -18153,7 +18818,7 @@
       </c>
       <c r="T128" s="2" t="inlineStr">
         <is>
-          <t>state unknown: source lists no location</t>
+          <t>state unknown: source lists no location; nces: skipped (state unknown)</t>
         </is>
       </c>
     </row>
@@ -18198,9 +18863,19 @@
         <v>2018</v>
       </c>
       <c r="J129" t="inlineStr"/>
-      <c r="K129" t="inlineStr"/>
-      <c r="L129" t="inlineStr"/>
-      <c r="M129" t="inlineStr"/>
+      <c r="K129" t="inlineStr">
+        <is>
+          <t>LINDBERGH SCHOOLS</t>
+        </is>
+      </c>
+      <c r="L129" t="n">
+        <v>2266</v>
+      </c>
+      <c r="M129" t="inlineStr">
+        <is>
+          <t>http://go.lindberghschools.ws/Domain/8</t>
+        </is>
+      </c>
       <c r="N129" t="inlineStr"/>
       <c r="O129" t="inlineStr"/>
       <c r="P129" t="inlineStr"/>
@@ -18211,7 +18886,11 @@
           <t>https://en.wikipedia.org/wiki/Rose_Parade_marching_bands</t>
         </is>
       </c>
-      <c r="T129" s="2" t="inlineStr"/>
+      <c r="T129" s="2" t="inlineStr">
+        <is>
+          <t>nces: matched 'LINDBERGH SR. HIGH' (0.92); site crawl blocked: HTTP 404 for http://go.lindberghschools.ws/Domain/8</t>
+        </is>
+      </c>
     </row>
     <row r="130">
       <c r="A130" t="inlineStr">
@@ -18254,9 +18933,19 @@
         <v>2018</v>
       </c>
       <c r="J130" t="inlineStr"/>
-      <c r="K130" t="inlineStr"/>
-      <c r="L130" t="inlineStr"/>
-      <c r="M130" t="inlineStr"/>
+      <c r="K130" t="inlineStr">
+        <is>
+          <t>Londonderry School District</t>
+        </is>
+      </c>
+      <c r="L130" t="n">
+        <v>1308</v>
+      </c>
+      <c r="M130" t="inlineStr">
+        <is>
+          <t>http://www.londonderry.org/lhs</t>
+        </is>
+      </c>
       <c r="N130" t="inlineStr"/>
       <c r="O130" t="inlineStr"/>
       <c r="P130" t="inlineStr"/>
@@ -18267,7 +18956,11 @@
           <t>https://en.wikipedia.org/wiki/Rose_Parade_marching_bands</t>
         </is>
       </c>
-      <c r="T130" s="2" t="inlineStr"/>
+      <c r="T130" s="2" t="inlineStr">
+        <is>
+          <t>site crawl blocked: HTTP 404 for http://www.londonderry.org/lhs</t>
+        </is>
+      </c>
     </row>
     <row r="131">
       <c r="A131" t="inlineStr">
@@ -18310,9 +19003,19 @@
         <v>2018</v>
       </c>
       <c r="J131" t="inlineStr"/>
-      <c r="K131" t="inlineStr"/>
-      <c r="L131" t="inlineStr"/>
-      <c r="M131" t="inlineStr"/>
+      <c r="K131" t="inlineStr">
+        <is>
+          <t>Louisburg</t>
+        </is>
+      </c>
+      <c r="L131" t="n">
+        <v>540</v>
+      </c>
+      <c r="M131" t="inlineStr">
+        <is>
+          <t>http://www.usd416.org</t>
+        </is>
+      </c>
       <c r="N131" t="inlineStr"/>
       <c r="O131" t="inlineStr"/>
       <c r="P131" t="inlineStr"/>
@@ -18323,7 +19026,11 @@
           <t>https://en.wikipedia.org/wiki/Rose_Parade_marching_bands</t>
         </is>
       </c>
-      <c r="T131" s="2" t="inlineStr"/>
+      <c r="T131" s="2" t="inlineStr">
+        <is>
+          <t>nces: matched 'Louisburg High' (0.92); no band page found in 1 pages crawled</t>
+        </is>
+      </c>
     </row>
     <row r="132">
       <c r="A132" t="inlineStr">
@@ -18369,7 +19076,7 @@
       </c>
       <c r="T132" s="2" t="inlineStr">
         <is>
-          <t>state unknown: source lists no location</t>
+          <t>state unknown: source lists no location; nces: skipped (state unknown)</t>
         </is>
       </c>
     </row>
@@ -18423,7 +19130,11 @@
           <t>https://en.wikipedia.org/wiki/Rose_Parade_marching_bands</t>
         </is>
       </c>
-      <c r="T133" s="2" t="inlineStr"/>
+      <c r="T133" s="2" t="inlineStr">
+        <is>
+          <t>nces: no match</t>
+        </is>
+      </c>
     </row>
     <row r="134">
       <c r="A134" t="inlineStr">
@@ -18466,8 +19177,14 @@
         <v>2015</v>
       </c>
       <c r="J134" t="inlineStr"/>
-      <c r="K134" t="inlineStr"/>
-      <c r="L134" t="inlineStr"/>
+      <c r="K134" t="inlineStr">
+        <is>
+          <t>Hawaii Department of Education</t>
+        </is>
+      </c>
+      <c r="L134" t="n">
+        <v>1908</v>
+      </c>
       <c r="M134" t="inlineStr"/>
       <c r="N134" t="inlineStr"/>
       <c r="O134" t="inlineStr"/>
@@ -18479,7 +19196,11 @@
           <t>https://en.wikipedia.org/wiki/Rose_Parade_marching_bands</t>
         </is>
       </c>
-      <c r="T134" s="2" t="inlineStr"/>
+      <c r="T134" s="2" t="inlineStr">
+        <is>
+          <t>no website in NCES</t>
+        </is>
+      </c>
     </row>
     <row r="135">
       <c r="A135" t="inlineStr">
@@ -18522,8 +19243,14 @@
         <v>2019</v>
       </c>
       <c r="J135" t="inlineStr"/>
-      <c r="K135" t="inlineStr"/>
-      <c r="L135" t="inlineStr"/>
+      <c r="K135" t="inlineStr">
+        <is>
+          <t>Mercer Island School District</t>
+        </is>
+      </c>
+      <c r="L135" t="n">
+        <v>1465</v>
+      </c>
       <c r="M135" t="inlineStr"/>
       <c r="N135" t="inlineStr"/>
       <c r="O135" t="inlineStr"/>
@@ -18535,7 +19262,11 @@
           <t>https://en.wikipedia.org/wiki/Rose_Parade_marching_bands</t>
         </is>
       </c>
-      <c r="T135" s="2" t="inlineStr"/>
+      <c r="T135" s="2" t="inlineStr">
+        <is>
+          <t>no website in NCES</t>
+        </is>
+      </c>
     </row>
     <row r="136">
       <c r="A136" t="inlineStr">
@@ -18585,7 +19316,7 @@
       </c>
       <c r="T136" s="2" t="inlineStr">
         <is>
-          <t>state unknown: source lists no location</t>
+          <t>state unknown: source lists no location; nces: skipped (state unknown)</t>
         </is>
       </c>
     </row>
@@ -18637,7 +19368,7 @@
       </c>
       <c r="T137" s="2" t="inlineStr">
         <is>
-          <t>state unknown: source lists no location</t>
+          <t>state unknown: source lists no location; nces: skipped (state unknown)</t>
         </is>
       </c>
     </row>
@@ -18689,7 +19420,7 @@
       </c>
       <c r="T138" s="2" t="inlineStr">
         <is>
-          <t>state unknown: source lists no location</t>
+          <t>state unknown: source lists no location; nces: skipped (state unknown)</t>
         </is>
       </c>
     </row>
@@ -18747,7 +19478,11 @@
           <t>https://en.wikipedia.org/wiki/Rose_Parade_marching_bands</t>
         </is>
       </c>
-      <c r="T139" s="2" t="inlineStr"/>
+      <c r="T139" s="2" t="inlineStr">
+        <is>
+          <t>nces: no match</t>
+        </is>
+      </c>
     </row>
     <row r="140">
       <c r="A140" t="inlineStr">
@@ -18799,7 +19534,11 @@
           <t>https://en.wikipedia.org/wiki/Rose_Parade_marching_bands</t>
         </is>
       </c>
-      <c r="T140" s="2" t="inlineStr"/>
+      <c r="T140" s="2" t="inlineStr">
+        <is>
+          <t>nces: no match</t>
+        </is>
+      </c>
     </row>
     <row r="141">
       <c r="A141" t="inlineStr">
@@ -18849,7 +19588,7 @@
       </c>
       <c r="T141" s="2" t="inlineStr">
         <is>
-          <t>state unknown: source lists no location</t>
+          <t>state unknown: source lists no location; nces: skipped (state unknown)</t>
         </is>
       </c>
     </row>
@@ -18907,7 +19646,11 @@
           <t>https://en.wikipedia.org/wiki/Rose_Parade_marching_bands</t>
         </is>
       </c>
-      <c r="T142" s="2" t="inlineStr"/>
+      <c r="T142" s="2" t="inlineStr">
+        <is>
+          <t>nces: no match</t>
+        </is>
+      </c>
     </row>
     <row r="143">
       <c r="A143" t="inlineStr">
@@ -19006,20 +19749,39 @@
         <v>2016</v>
       </c>
       <c r="J144" t="inlineStr"/>
-      <c r="K144" t="inlineStr"/>
-      <c r="L144" t="inlineStr"/>
-      <c r="M144" t="inlineStr"/>
-      <c r="N144" t="inlineStr"/>
+      <c r="K144" t="inlineStr">
+        <is>
+          <t>Los Gatos-Saratoga Union High</t>
+        </is>
+      </c>
+      <c r="L144" t="n">
+        <v>1198</v>
+      </c>
+      <c r="M144" t="inlineStr">
+        <is>
+          <t>http://www.saratogahigh.org</t>
+        </is>
+      </c>
+      <c r="N144" t="inlineStr">
+        <is>
+          <t>https://www.saratogamusicboosters.org/</t>
+        </is>
+      </c>
       <c r="O144" t="inlineStr"/>
       <c r="P144" t="inlineStr"/>
       <c r="Q144" t="inlineStr"/>
       <c r="R144" t="inlineStr"/>
       <c r="S144" s="2" t="inlineStr">
         <is>
-          <t>https://en.wikipedia.org/wiki/Rose_Parade_marching_bands</t>
-        </is>
-      </c>
-      <c r="T144" s="2" t="inlineStr"/>
+          <t>https://en.wikipedia.org/wiki/Rose_Parade_marching_bands
+https://www.saratogamusicboosters.org/</t>
+        </is>
+      </c>
+      <c r="T144" s="2" t="inlineStr">
+        <is>
+          <t>nces: matched 'Saratoga High' (0.92); social: https://www.instagram.com/saratogamusicboosters; social: https://www.facebook.com/saratogamusicboosters; social: https://www.instagram.com/reel/CxUE6_IpT2c</t>
+        </is>
+      </c>
     </row>
     <row r="145">
       <c r="A145" t="inlineStr">
@@ -19065,7 +19827,7 @@
       </c>
       <c r="T145" s="2" t="inlineStr">
         <is>
-          <t>state unknown: source lists no location</t>
+          <t>state unknown: source lists no location; nces: skipped (state unknown)</t>
         </is>
       </c>
     </row>
@@ -19110,8 +19872,14 @@
         <v>2015</v>
       </c>
       <c r="J146" t="inlineStr"/>
-      <c r="K146" t="inlineStr"/>
-      <c r="L146" t="inlineStr"/>
+      <c r="K146" t="inlineStr">
+        <is>
+          <t>Temple City Unified</t>
+        </is>
+      </c>
+      <c r="L146" t="n">
+        <v>1758</v>
+      </c>
       <c r="M146" t="inlineStr"/>
       <c r="N146" t="inlineStr"/>
       <c r="O146" t="inlineStr"/>
@@ -19123,7 +19891,11 @@
           <t>https://en.wikipedia.org/wiki/Rose_Parade_marching_bands</t>
         </is>
       </c>
-      <c r="T146" s="2" t="inlineStr"/>
+      <c r="T146" s="2" t="inlineStr">
+        <is>
+          <t>nces: matched 'Temple City High' (0.92); no website in NCES</t>
+        </is>
+      </c>
     </row>
     <row r="147">
       <c r="A147" t="inlineStr">
@@ -19175,7 +19947,11 @@
           <t>https://en.wikipedia.org/wiki/Rose_Parade_marching_bands</t>
         </is>
       </c>
-      <c r="T147" s="2" t="inlineStr"/>
+      <c r="T147" s="2" t="inlineStr">
+        <is>
+          <t>nces: no match</t>
+        </is>
+      </c>
     </row>
     <row r="148">
       <c r="A148" t="inlineStr">
@@ -19218,9 +19994,19 @@
         <v>2018</v>
       </c>
       <c r="J148" t="inlineStr"/>
-      <c r="K148" t="inlineStr"/>
-      <c r="L148" t="inlineStr"/>
-      <c r="M148" t="inlineStr"/>
+      <c r="K148" t="inlineStr">
+        <is>
+          <t>Alpine District</t>
+        </is>
+      </c>
+      <c r="L148" t="n">
+        <v>2847</v>
+      </c>
+      <c r="M148" t="inlineStr">
+        <is>
+          <t>http://westlake.alpinedistrict.org/</t>
+        </is>
+      </c>
       <c r="N148" t="inlineStr"/>
       <c r="O148" t="inlineStr"/>
       <c r="P148" t="inlineStr"/>
@@ -19231,7 +20017,11 @@
           <t>https://en.wikipedia.org/wiki/Rose_Parade_marching_bands</t>
         </is>
       </c>
-      <c r="T148" s="2" t="inlineStr"/>
+      <c r="T148" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">nces: matched 'Westlake High' (0.92); site crawl blocked: TLS failure for http://westlake.alpinedistrict.org/: HTTPSConnectionPool(host='westlake.alpinedistrict.org', port=443): </t>
+        </is>
+      </c>
     </row>
     <row r="149">
       <c r="A149" t="inlineStr">
@@ -19336,9 +20126,19 @@
         <v>2019</v>
       </c>
       <c r="J150" t="inlineStr"/>
-      <c r="K150" t="inlineStr"/>
-      <c r="L150" t="inlineStr"/>
-      <c r="M150" t="inlineStr"/>
+      <c r="K150" t="inlineStr">
+        <is>
+          <t>Decatur County</t>
+        </is>
+      </c>
+      <c r="L150" t="n">
+        <v>1218</v>
+      </c>
+      <c r="M150" t="inlineStr">
+        <is>
+          <t>http://bhs.boe.dcboe.com/</t>
+        </is>
+      </c>
       <c r="N150" t="inlineStr"/>
       <c r="O150" t="inlineStr"/>
       <c r="P150" t="inlineStr"/>
@@ -19349,7 +20149,11 @@
           <t>https://en.wikipedia.org/wiki/6abc_Dunkin%27_Thanksgiving_Day_Parade</t>
         </is>
       </c>
-      <c r="T150" s="2" t="inlineStr"/>
+      <c r="T150" s="2" t="inlineStr">
+        <is>
+          <t>no band page found in 1 pages crawled</t>
+        </is>
+      </c>
     </row>
     <row r="151">
       <c r="A151" t="inlineStr">
@@ -19392,9 +20196,19 @@
         <v>2016</v>
       </c>
       <c r="J151" t="inlineStr"/>
-      <c r="K151" t="inlineStr"/>
-      <c r="L151" t="inlineStr"/>
-      <c r="M151" t="inlineStr"/>
+      <c r="K151" t="inlineStr">
+        <is>
+          <t>Lauderdale County</t>
+        </is>
+      </c>
+      <c r="L151" t="n">
+        <v>744</v>
+      </c>
+      <c r="M151" t="inlineStr">
+        <is>
+          <t>http://www.lcschools.org</t>
+        </is>
+      </c>
       <c r="N151" t="inlineStr"/>
       <c r="O151" t="inlineStr"/>
       <c r="P151" t="inlineStr"/>
@@ -19405,7 +20219,11 @@
           <t>https://en.wikipedia.org/wiki/6abc_Dunkin%27_Thanksgiving_Day_Parade</t>
         </is>
       </c>
-      <c r="T151" s="2" t="inlineStr"/>
+      <c r="T151" s="2" t="inlineStr">
+        <is>
+          <t>no band page found in 1 pages crawled</t>
+        </is>
+      </c>
     </row>
     <row r="152">
       <c r="A152" t="inlineStr">
@@ -19444,8 +20262,14 @@
         <v>2019</v>
       </c>
       <c r="J152" t="inlineStr"/>
-      <c r="K152" t="inlineStr"/>
-      <c r="L152" t="inlineStr"/>
+      <c r="K152" t="inlineStr">
+        <is>
+          <t>Glynn County</t>
+        </is>
+      </c>
+      <c r="L152" t="n">
+        <v>1939</v>
+      </c>
       <c r="M152" t="inlineStr"/>
       <c r="N152" t="inlineStr"/>
       <c r="O152" t="inlineStr"/>
@@ -19457,7 +20281,11 @@
           <t>https://en.wikipedia.org/wiki/6abc_Dunkin%27_Thanksgiving_Day_Parade</t>
         </is>
       </c>
-      <c r="T152" s="2" t="inlineStr"/>
+      <c r="T152" s="2" t="inlineStr">
+        <is>
+          <t>nces: matched 'Brunswick High School' (0.92); no website in NCES</t>
+        </is>
+      </c>
     </row>
     <row r="153">
       <c r="A153" t="inlineStr">
@@ -19570,9 +20398,19 @@
         <v>2019</v>
       </c>
       <c r="J154" t="inlineStr"/>
-      <c r="K154" t="inlineStr"/>
-      <c r="L154" t="inlineStr"/>
-      <c r="M154" t="inlineStr"/>
+      <c r="K154" t="inlineStr">
+        <is>
+          <t>Colquitt County</t>
+        </is>
+      </c>
+      <c r="L154" t="n">
+        <v>1871</v>
+      </c>
+      <c r="M154" t="inlineStr">
+        <is>
+          <t>http://colquitt.k12.ga.us/cchs/</t>
+        </is>
+      </c>
       <c r="N154" t="inlineStr"/>
       <c r="O154" t="inlineStr"/>
       <c r="P154" t="inlineStr"/>
@@ -19583,7 +20421,11 @@
           <t>https://en.wikipedia.org/wiki/6abc_Dunkin%27_Thanksgiving_Day_Parade</t>
         </is>
       </c>
-      <c r="T154" s="2" t="inlineStr"/>
+      <c r="T154" s="2" t="inlineStr">
+        <is>
+          <t>site crawl blocked: TLS failure for http://colquitt.k12.ga.us/cchs/: HTTPSConnectionPool(host='www.colquitt.k12.ga.us', port=443): Max retri</t>
+        </is>
+      </c>
     </row>
     <row r="155">
       <c r="A155" t="inlineStr">
@@ -19678,9 +20520,19 @@
         <v>2019</v>
       </c>
       <c r="J156" t="inlineStr"/>
-      <c r="K156" t="inlineStr"/>
-      <c r="L156" t="inlineStr"/>
-      <c r="M156" t="inlineStr"/>
+      <c r="K156" t="inlineStr">
+        <is>
+          <t>Guntersville City</t>
+        </is>
+      </c>
+      <c r="L156" t="n">
+        <v>523</v>
+      </c>
+      <c r="M156" t="inlineStr">
+        <is>
+          <t>http://www.guntersville-high.com</t>
+        </is>
+      </c>
       <c r="N156" t="inlineStr"/>
       <c r="O156" t="inlineStr"/>
       <c r="P156" t="inlineStr"/>
@@ -19691,7 +20543,11 @@
           <t>https://en.wikipedia.org/wiki/6abc_Dunkin%27_Thanksgiving_Day_Parade</t>
         </is>
       </c>
-      <c r="T156" s="2" t="inlineStr"/>
+      <c r="T156" s="2" t="inlineStr">
+        <is>
+          <t>site crawl blocked: HTTP 503 for http://www.guntersville-high.com</t>
+        </is>
+      </c>
     </row>
     <row r="157">
       <c r="A157" t="inlineStr">
@@ -19734,9 +20590,19 @@
         <v>2016</v>
       </c>
       <c r="J157" t="inlineStr"/>
-      <c r="K157" t="inlineStr"/>
-      <c r="L157" t="inlineStr"/>
-      <c r="M157" t="inlineStr"/>
+      <c r="K157" t="inlineStr">
+        <is>
+          <t>Huntsville City</t>
+        </is>
+      </c>
+      <c r="L157" t="n">
+        <v>1802</v>
+      </c>
+      <c r="M157" t="inlineStr">
+        <is>
+          <t>http://www.huntsvillecityschools.org</t>
+        </is>
+      </c>
       <c r="N157" t="inlineStr"/>
       <c r="O157" t="inlineStr"/>
       <c r="P157" t="inlineStr"/>
@@ -19747,7 +20613,11 @@
           <t>https://en.wikipedia.org/wiki/6abc_Dunkin%27_Thanksgiving_Day_Parade</t>
         </is>
       </c>
-      <c r="T157" s="2" t="inlineStr"/>
+      <c r="T157" s="2" t="inlineStr">
+        <is>
+          <t>no band page found in 1 pages crawled</t>
+        </is>
+      </c>
     </row>
     <row r="158">
       <c r="A158" t="inlineStr">
@@ -19879,7 +20749,11 @@
           <t>https://en.wikipedia.org/wiki/6abc_Dunkin%27_Thanksgiving_Day_Parade</t>
         </is>
       </c>
-      <c r="T159" s="2" t="inlineStr"/>
+      <c r="T159" s="2" t="inlineStr">
+        <is>
+          <t>no band page found in 7 pages crawled</t>
+        </is>
+      </c>
     </row>
     <row r="160">
       <c r="A160" t="inlineStr">
@@ -19918,9 +20792,19 @@
         <v>2018</v>
       </c>
       <c r="J160" t="inlineStr"/>
-      <c r="K160" t="inlineStr"/>
-      <c r="L160" t="inlineStr"/>
-      <c r="M160" t="inlineStr"/>
+      <c r="K160" t="inlineStr">
+        <is>
+          <t>Lowndes County</t>
+        </is>
+      </c>
+      <c r="L160" t="n">
+        <v>3210</v>
+      </c>
+      <c r="M160" t="inlineStr">
+        <is>
+          <t>http://lhs.lowndes.k12.ga.us/</t>
+        </is>
+      </c>
       <c r="N160" t="inlineStr"/>
       <c r="O160" t="inlineStr"/>
       <c r="P160" t="inlineStr"/>
@@ -19931,7 +20815,11 @@
           <t>https://en.wikipedia.org/wiki/6abc_Dunkin%27_Thanksgiving_Day_Parade</t>
         </is>
       </c>
-      <c r="T160" s="2" t="inlineStr"/>
+      <c r="T160" s="2" t="inlineStr">
+        <is>
+          <t>nces: matched 'Lowndes High School' (0.92); no band page found in 1 pages crawled</t>
+        </is>
+      </c>
     </row>
     <row r="161">
       <c r="A161" t="inlineStr">
@@ -19974,9 +20862,19 @@
         <v>2019</v>
       </c>
       <c r="J161" t="inlineStr"/>
-      <c r="K161" t="inlineStr"/>
-      <c r="L161" t="inlineStr"/>
-      <c r="M161" t="inlineStr"/>
+      <c r="K161" t="inlineStr">
+        <is>
+          <t>Mobile County</t>
+        </is>
+      </c>
+      <c r="L161" t="n">
+        <v>1918</v>
+      </c>
+      <c r="M161" t="inlineStr">
+        <is>
+          <t>http://montgomery.mcs.schoolinsites.com</t>
+        </is>
+      </c>
       <c r="N161" t="inlineStr"/>
       <c r="O161" t="inlineStr"/>
       <c r="P161" t="inlineStr"/>
@@ -19987,7 +20885,11 @@
           <t>https://en.wikipedia.org/wiki/6abc_Dunkin%27_Thanksgiving_Day_Parade</t>
         </is>
       </c>
-      <c r="T161" s="2" t="inlineStr"/>
+      <c r="T161" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">site crawl blocked: request failed for http://montgomery.mcs.schoolinsites.com: HTTPConnectionPool(host='montgomery.mcs.schoolinsites.com', </t>
+        </is>
+      </c>
     </row>
     <row r="162">
       <c r="A162" t="inlineStr">
@@ -20096,8 +20998,14 @@
         <v>2016</v>
       </c>
       <c r="J163" t="inlineStr"/>
-      <c r="K163" t="inlineStr"/>
-      <c r="L163" t="inlineStr"/>
+      <c r="K163" t="inlineStr">
+        <is>
+          <t>Aiken 01</t>
+        </is>
+      </c>
+      <c r="L163" t="n">
+        <v>1697</v>
+      </c>
       <c r="M163" t="inlineStr"/>
       <c r="N163" t="inlineStr"/>
       <c r="O163" t="inlineStr"/>
@@ -20109,7 +21017,11 @@
           <t>https://en.wikipedia.org/wiki/6abc_Dunkin%27_Thanksgiving_Day_Parade</t>
         </is>
       </c>
-      <c r="T163" s="2" t="inlineStr"/>
+      <c r="T163" s="2" t="inlineStr">
+        <is>
+          <t>nces: matched 'North Augusta High' (0.92); no website in NCES</t>
+        </is>
+      </c>
     </row>
     <row r="164">
       <c r="A164" t="inlineStr">
@@ -20152,9 +21064,19 @@
         <v>2015</v>
       </c>
       <c r="J164" t="inlineStr"/>
-      <c r="K164" t="inlineStr"/>
-      <c r="L164" t="inlineStr"/>
-      <c r="M164" t="inlineStr"/>
+      <c r="K164" t="inlineStr">
+        <is>
+          <t>Oneonta City</t>
+        </is>
+      </c>
+      <c r="L164" t="n">
+        <v>428</v>
+      </c>
+      <c r="M164" t="inlineStr">
+        <is>
+          <t>http://www.oneontacityschools.com</t>
+        </is>
+      </c>
       <c r="N164" t="inlineStr"/>
       <c r="O164" t="inlineStr"/>
       <c r="P164" t="inlineStr"/>
@@ -20165,7 +21087,11 @@
           <t>https://en.wikipedia.org/wiki/6abc_Dunkin%27_Thanksgiving_Day_Parade</t>
         </is>
       </c>
-      <c r="T164" s="2" t="inlineStr"/>
+      <c r="T164" s="2" t="inlineStr">
+        <is>
+          <t>no band page found in 1 pages crawled</t>
+        </is>
+      </c>
     </row>
     <row r="165">
       <c r="A165" t="inlineStr">
@@ -20208,17 +21134,32 @@
         <v>2022</v>
       </c>
       <c r="J165" t="inlineStr"/>
-      <c r="K165" t="inlineStr"/>
-      <c r="L165" t="inlineStr"/>
-      <c r="M165" t="inlineStr"/>
-      <c r="N165" t="inlineStr"/>
+      <c r="K165" t="inlineStr">
+        <is>
+          <t>Parkland SD</t>
+        </is>
+      </c>
+      <c r="L165" t="n">
+        <v>3242</v>
+      </c>
+      <c r="M165" t="inlineStr">
+        <is>
+          <t>http://phs.parklandsd.org/</t>
+        </is>
+      </c>
+      <c r="N165" t="inlineStr">
+        <is>
+          <t>http://phs.parklandsd.org/departments/music</t>
+        </is>
+      </c>
       <c r="O165" t="inlineStr"/>
       <c r="P165" t="inlineStr"/>
       <c r="Q165" t="inlineStr"/>
       <c r="R165" t="inlineStr"/>
       <c r="S165" s="2" t="inlineStr">
         <is>
-          <t>https://en.wikipedia.org/wiki/6abc_Dunkin%27_Thanksgiving_Day_Parade</t>
+          <t>https://en.wikipedia.org/wiki/6abc_Dunkin%27_Thanksgiving_Day_Parade
+http://phs.parklandsd.org/departments/music</t>
         </is>
       </c>
       <c r="T165" s="2" t="inlineStr"/>
@@ -20277,7 +21218,11 @@
           <t>https://en.wikipedia.org/wiki/6abc_Dunkin%27_Thanksgiving_Day_Parade</t>
         </is>
       </c>
-      <c r="T166" s="2" t="inlineStr"/>
+      <c r="T166" s="2" t="inlineStr">
+        <is>
+          <t>nces: no match</t>
+        </is>
+      </c>
     </row>
     <row r="167">
       <c r="A167" t="inlineStr">
@@ -20320,8 +21265,14 @@
         <v>2022</v>
       </c>
       <c r="J167" t="inlineStr"/>
-      <c r="K167" t="inlineStr"/>
-      <c r="L167" t="inlineStr"/>
+      <c r="K167" t="inlineStr">
+        <is>
+          <t>Pocono Mountain SD</t>
+        </is>
+      </c>
+      <c r="L167" t="n">
+        <v>1256</v>
+      </c>
       <c r="M167" t="inlineStr"/>
       <c r="N167" t="inlineStr"/>
       <c r="O167" t="inlineStr"/>
@@ -20333,7 +21284,11 @@
           <t>https://en.wikipedia.org/wiki/6abc_Dunkin%27_Thanksgiving_Day_Parade</t>
         </is>
       </c>
-      <c r="T167" s="2" t="inlineStr"/>
+      <c r="T167" s="2" t="inlineStr">
+        <is>
+          <t>no website in NCES</t>
+        </is>
+      </c>
     </row>
     <row r="168">
       <c r="A168" t="inlineStr">
@@ -20372,8 +21327,14 @@
         <v>2022</v>
       </c>
       <c r="J168" t="inlineStr"/>
-      <c r="K168" t="inlineStr"/>
-      <c r="L168" t="inlineStr"/>
+      <c r="K168" t="inlineStr">
+        <is>
+          <t>Reynoldsburg City</t>
+        </is>
+      </c>
+      <c r="L168" t="n">
+        <v>2268</v>
+      </c>
       <c r="M168" t="inlineStr"/>
       <c r="N168" t="inlineStr"/>
       <c r="O168" t="inlineStr"/>
@@ -20385,7 +21346,11 @@
           <t>https://en.wikipedia.org/wiki/6abc_Dunkin%27_Thanksgiving_Day_Parade</t>
         </is>
       </c>
-      <c r="T168" s="2" t="inlineStr"/>
+      <c r="T168" s="2" t="inlineStr">
+        <is>
+          <t>nces: matched 'Reynoldsburg High School' (0.92); no website in NCES</t>
+        </is>
+      </c>
     </row>
     <row r="169">
       <c r="A169" t="inlineStr">
@@ -20428,9 +21393,19 @@
         <v>2016</v>
       </c>
       <c r="J169" t="inlineStr"/>
-      <c r="K169" t="inlineStr"/>
-      <c r="L169" t="inlineStr"/>
-      <c r="M169" t="inlineStr"/>
+      <c r="K169" t="inlineStr">
+        <is>
+          <t>Rome City</t>
+        </is>
+      </c>
+      <c r="L169" t="n">
+        <v>2015</v>
+      </c>
+      <c r="M169" t="inlineStr">
+        <is>
+          <t>http://www.rcs.rome.ga.us</t>
+        </is>
+      </c>
       <c r="N169" t="inlineStr"/>
       <c r="O169" t="inlineStr"/>
       <c r="P169" t="inlineStr"/>
@@ -20441,7 +21416,11 @@
           <t>https://en.wikipedia.org/wiki/6abc_Dunkin%27_Thanksgiving_Day_Parade</t>
         </is>
       </c>
-      <c r="T169" s="2" t="inlineStr"/>
+      <c r="T169" s="2" t="inlineStr">
+        <is>
+          <t>no band page found in 1 pages crawled</t>
+        </is>
+      </c>
     </row>
     <row r="170">
       <c r="A170" t="inlineStr">
@@ -20484,9 +21463,19 @@
         <v>2015</v>
       </c>
       <c r="J170" t="inlineStr"/>
-      <c r="K170" t="inlineStr"/>
-      <c r="L170" t="inlineStr"/>
-      <c r="M170" t="inlineStr"/>
+      <c r="K170" t="inlineStr">
+        <is>
+          <t>Lee County</t>
+        </is>
+      </c>
+      <c r="L170" t="n">
+        <v>1222</v>
+      </c>
+      <c r="M170" t="inlineStr">
+        <is>
+          <t>http://www.lee.k12.al.us</t>
+        </is>
+      </c>
       <c r="N170" t="inlineStr"/>
       <c r="O170" t="inlineStr"/>
       <c r="P170" t="inlineStr"/>
@@ -20497,7 +21486,11 @@
           <t>https://en.wikipedia.org/wiki/6abc_Dunkin%27_Thanksgiving_Day_Parade</t>
         </is>
       </c>
-      <c r="T170" s="2" t="inlineStr"/>
+      <c r="T170" s="2" t="inlineStr">
+        <is>
+          <t>no band page found in 1 pages crawled</t>
+        </is>
+      </c>
     </row>
     <row r="171">
       <c r="A171" t="inlineStr">
@@ -20514,7 +21507,11 @@
         </is>
       </c>
       <c r="D171" t="inlineStr"/>
-      <c r="E171" t="inlineStr"/>
+      <c r="E171" t="inlineStr">
+        <is>
+          <t>Austin</t>
+        </is>
+      </c>
       <c r="F171" t="inlineStr">
         <is>
           <t>TX</t>
@@ -20536,8 +21533,14 @@
           <t>2019</t>
         </is>
       </c>
-      <c r="K171" t="inlineStr"/>
-      <c r="L171" t="inlineStr"/>
+      <c r="K171" t="inlineStr">
+        <is>
+          <t>LEANDER ISD</t>
+        </is>
+      </c>
+      <c r="L171" t="n">
+        <v>2522</v>
+      </c>
       <c r="M171" t="inlineStr"/>
       <c r="N171" t="inlineStr"/>
       <c r="O171" t="inlineStr"/>
@@ -20549,7 +21552,11 @@
           <t>https://marching.musicforall.org/result/grand-national-championships/</t>
         </is>
       </c>
-      <c r="T171" s="2" t="inlineStr"/>
+      <c r="T171" s="2" t="inlineStr">
+        <is>
+          <t>no website in NCES</t>
+        </is>
+      </c>
     </row>
     <row r="172">
       <c r="A172" t="inlineStr">
@@ -20592,9 +21599,19 @@
         <v>2016</v>
       </c>
       <c r="J172" t="inlineStr"/>
-      <c r="K172" t="inlineStr"/>
-      <c r="L172" t="inlineStr"/>
-      <c r="M172" t="inlineStr"/>
+      <c r="K172" t="inlineStr">
+        <is>
+          <t>Wayne County</t>
+        </is>
+      </c>
+      <c r="L172" t="n">
+        <v>1509</v>
+      </c>
+      <c r="M172" t="inlineStr">
+        <is>
+          <t>http://www.wayne.k12.ga.us</t>
+        </is>
+      </c>
       <c r="N172" t="inlineStr"/>
       <c r="O172" t="inlineStr"/>
       <c r="P172" t="inlineStr"/>
@@ -20605,7 +21622,11 @@
           <t>https://en.wikipedia.org/wiki/6abc_Dunkin%27_Thanksgiving_Day_Parade</t>
         </is>
       </c>
-      <c r="T172" s="2" t="inlineStr"/>
+      <c r="T172" s="2" t="inlineStr">
+        <is>
+          <t>no band page found in 1 pages crawled</t>
+        </is>
+      </c>
     </row>
     <row r="173">
       <c r="A173" t="inlineStr">
@@ -20648,8 +21669,14 @@
         <v>2019</v>
       </c>
       <c r="J173" t="inlineStr"/>
-      <c r="K173" t="inlineStr"/>
-      <c r="L173" t="inlineStr"/>
+      <c r="K173" t="inlineStr">
+        <is>
+          <t>Lexington 01</t>
+        </is>
+      </c>
+      <c r="L173" t="n">
+        <v>2031</v>
+      </c>
       <c r="M173" t="inlineStr"/>
       <c r="N173" t="inlineStr"/>
       <c r="O173" t="inlineStr"/>
@@ -20661,7 +21688,11 @@
           <t>https://en.wikipedia.org/wiki/6abc_Dunkin%27_Thanksgiving_Day_Parade</t>
         </is>
       </c>
-      <c r="T173" s="2" t="inlineStr"/>
+      <c r="T173" s="2" t="inlineStr">
+        <is>
+          <t>nces: matched 'White Knoll High' (0.92); no website in NCES</t>
+        </is>
+      </c>
     </row>
     <row r="174">
       <c r="A174" t="inlineStr">
@@ -20770,9 +21801,19 @@
         <v>2016</v>
       </c>
       <c r="J175" t="inlineStr"/>
-      <c r="K175" t="inlineStr"/>
-      <c r="L175" t="inlineStr"/>
-      <c r="M175" t="inlineStr"/>
+      <c r="K175" t="inlineStr">
+        <is>
+          <t>Henry County</t>
+        </is>
+      </c>
+      <c r="L175" t="n">
+        <v>1322</v>
+      </c>
+      <c r="M175" t="inlineStr">
+        <is>
+          <t>http://www.henry.k12.ga.us/wh</t>
+        </is>
+      </c>
       <c r="N175" t="inlineStr"/>
       <c r="O175" t="inlineStr"/>
       <c r="P175" t="inlineStr"/>
@@ -20783,7 +21824,11 @@
           <t>https://en.wikipedia.org/wiki/6abc_Dunkin%27_Thanksgiving_Day_Parade</t>
         </is>
       </c>
-      <c r="T175" s="2" t="inlineStr"/>
+      <c r="T175" s="2" t="inlineStr">
+        <is>
+          <t>site crawl blocked: HTTP 404 for http://www.henry.k12.ga.us/wh</t>
+        </is>
+      </c>
     </row>
     <row r="176">
       <c r="A176" t="inlineStr">
@@ -20835,7 +21880,11 @@
           <t>https://marching.musicforall.org/result/grand-national-championships/</t>
         </is>
       </c>
-      <c r="T176" s="2" t="inlineStr"/>
+      <c r="T176" s="2" t="inlineStr">
+        <is>
+          <t>nces: no match</t>
+        </is>
+      </c>
     </row>
     <row r="177">
       <c r="A177" t="inlineStr">
@@ -20878,9 +21927,19 @@
         <v>2018</v>
       </c>
       <c r="J177" t="inlineStr"/>
-      <c r="K177" t="inlineStr"/>
-      <c r="L177" t="inlineStr"/>
-      <c r="M177" t="inlineStr"/>
+      <c r="K177" t="inlineStr">
+        <is>
+          <t>BILOXI PUBLIC SCHOOL DIST</t>
+        </is>
+      </c>
+      <c r="L177" t="n">
+        <v>1697</v>
+      </c>
+      <c r="M177" t="inlineStr">
+        <is>
+          <t>http://www.biloxischools.net</t>
+        </is>
+      </c>
       <c r="N177" t="inlineStr"/>
       <c r="O177" t="inlineStr"/>
       <c r="P177" t="inlineStr"/>
@@ -20891,7 +21950,11 @@
           <t>https://en.wikipedia.org/wiki/6abc_Dunkin%27_Thanksgiving_Day_Parade</t>
         </is>
       </c>
-      <c r="T177" s="2" t="inlineStr"/>
+      <c r="T177" s="2" t="inlineStr">
+        <is>
+          <t>no band page found in 4 pages crawled</t>
+        </is>
+      </c>
     </row>
     <row r="178">
       <c r="A178" t="inlineStr">
@@ -20943,7 +22006,11 @@
           <t>https://en.wikipedia.org/wiki/6abc_Dunkin%27_Thanksgiving_Day_Parade</t>
         </is>
       </c>
-      <c r="T178" s="2" t="inlineStr"/>
+      <c r="T178" s="2" t="inlineStr">
+        <is>
+          <t>nces: no match</t>
+        </is>
+      </c>
     </row>
     <row r="179">
       <c r="A179" t="inlineStr">
@@ -20986,8 +22053,14 @@
         <v>2019</v>
       </c>
       <c r="J179" t="inlineStr"/>
-      <c r="K179" t="inlineStr"/>
-      <c r="L179" t="inlineStr"/>
+      <c r="K179" t="inlineStr">
+        <is>
+          <t>MONONGALIA COUNTY SCHOOLS</t>
+        </is>
+      </c>
+      <c r="L179" t="n">
+        <v>1824</v>
+      </c>
       <c r="M179" t="inlineStr"/>
       <c r="N179" t="inlineStr"/>
       <c r="O179" t="inlineStr"/>
@@ -20999,7 +22072,11 @@
           <t>https://en.wikipedia.org/wiki/6abc_Dunkin%27_Thanksgiving_Day_Parade</t>
         </is>
       </c>
-      <c r="T179" s="2" t="inlineStr"/>
+      <c r="T179" s="2" t="inlineStr">
+        <is>
+          <t>no website in NCES</t>
+        </is>
+      </c>
     </row>
     <row r="180">
       <c r="A180" t="inlineStr">
@@ -21016,7 +22093,11 @@
         </is>
       </c>
       <c r="D180" t="inlineStr"/>
-      <c r="E180" t="inlineStr"/>
+      <c r="E180" t="inlineStr">
+        <is>
+          <t>Tulsa</t>
+        </is>
+      </c>
       <c r="F180" t="inlineStr">
         <is>
           <t>OK</t>
@@ -21038,20 +22119,39 @@
           <t>2019</t>
         </is>
       </c>
-      <c r="K180" t="inlineStr"/>
-      <c r="L180" t="inlineStr"/>
-      <c r="M180" t="inlineStr"/>
-      <c r="N180" t="inlineStr"/>
+      <c r="K180" t="inlineStr">
+        <is>
+          <t>UNION</t>
+        </is>
+      </c>
+      <c r="L180" t="n">
+        <v>3516</v>
+      </c>
+      <c r="M180" t="inlineStr">
+        <is>
+          <t>http://www.unionps.org/</t>
+        </is>
+      </c>
+      <c r="N180" t="inlineStr">
+        <is>
+          <t>http://www.unionps.org/</t>
+        </is>
+      </c>
       <c r="O180" t="inlineStr"/>
       <c r="P180" t="inlineStr"/>
       <c r="Q180" t="inlineStr"/>
       <c r="R180" t="inlineStr"/>
       <c r="S180" s="2" t="inlineStr">
         <is>
-          <t>https://marching.musicforall.org/result/grand-national-championships/</t>
-        </is>
-      </c>
-      <c r="T180" s="2" t="inlineStr"/>
+          <t>https://marching.musicforall.org/result/grand-national-championships/
+http://www.unionps.org/</t>
+        </is>
+      </c>
+      <c r="T180" s="2" t="inlineStr">
+        <is>
+          <t>social: https://www.facebook.com/UnionSchools; social: https://www.instagram.com/unionschools</t>
+        </is>
+      </c>
     </row>
     <row r="181">
       <c r="A181" t="inlineStr">
@@ -21103,7 +22203,11 @@
           <t>https://en.wikipedia.org/wiki/6abc_Dunkin%27_Thanksgiving_Day_Parade</t>
         </is>
       </c>
-      <c r="T181" s="2" t="inlineStr"/>
+      <c r="T181" s="2" t="inlineStr">
+        <is>
+          <t>nces: no match</t>
+        </is>
+      </c>
     </row>
     <row r="182">
       <c r="A182" t="inlineStr">
@@ -21155,7 +22259,11 @@
           <t>https://en.wikipedia.org/wiki/6abc_Dunkin%27_Thanksgiving_Day_Parade</t>
         </is>
       </c>
-      <c r="T182" s="2" t="inlineStr"/>
+      <c r="T182" s="2" t="inlineStr">
+        <is>
+          <t>nces: no match</t>
+        </is>
+      </c>
     </row>
     <row r="183">
       <c r="A183" t="inlineStr">
@@ -21198,8 +22306,14 @@
         <v>2016</v>
       </c>
       <c r="J183" t="inlineStr"/>
-      <c r="K183" t="inlineStr"/>
-      <c r="L183" t="inlineStr"/>
+      <c r="K183" t="inlineStr">
+        <is>
+          <t>Anthony Wayne Local</t>
+        </is>
+      </c>
+      <c r="L183" t="n">
+        <v>1335</v>
+      </c>
       <c r="M183" t="inlineStr"/>
       <c r="N183" t="inlineStr"/>
       <c r="O183" t="inlineStr"/>
@@ -21211,7 +22325,11 @@
           <t>https://en.wikipedia.org/wiki/6abc_Dunkin%27_Thanksgiving_Day_Parade</t>
         </is>
       </c>
-      <c r="T183" s="2" t="inlineStr"/>
+      <c r="T183" s="2" t="inlineStr">
+        <is>
+          <t>no website in NCES</t>
+        </is>
+      </c>
     </row>
     <row r="184">
       <c r="A184" t="inlineStr">
@@ -21263,7 +22381,11 @@
           <t>https://en.wikipedia.org/wiki/6abc_Dunkin%27_Thanksgiving_Day_Parade</t>
         </is>
       </c>
-      <c r="T184" s="2" t="inlineStr"/>
+      <c r="T184" s="2" t="inlineStr">
+        <is>
+          <t>nces: no match</t>
+        </is>
+      </c>
     </row>
     <row r="185">
       <c r="A185" t="inlineStr">
@@ -21315,7 +22437,11 @@
           <t>https://en.wikipedia.org/wiki/6abc_Dunkin%27_Thanksgiving_Day_Parade</t>
         </is>
       </c>
-      <c r="T185" s="2" t="inlineStr"/>
+      <c r="T185" s="2" t="inlineStr">
+        <is>
+          <t>nces: no match</t>
+        </is>
+      </c>
     </row>
     <row r="186">
       <c r="A186" t="inlineStr">
@@ -21361,7 +22487,7 @@
       </c>
       <c r="T186" s="2" t="inlineStr">
         <is>
-          <t>state unknown: source lists no location</t>
+          <t>state unknown: source lists no location; nces: skipped (state unknown)</t>
         </is>
       </c>
     </row>
@@ -21406,8 +22532,14 @@
         <v>2018</v>
       </c>
       <c r="J187" t="inlineStr"/>
-      <c r="K187" t="inlineStr"/>
-      <c r="L187" t="inlineStr"/>
+      <c r="K187" t="inlineStr">
+        <is>
+          <t>Monroe County Community Sch Corp</t>
+        </is>
+      </c>
+      <c r="L187" t="n">
+        <v>1562</v>
+      </c>
       <c r="M187" t="inlineStr"/>
       <c r="N187" t="inlineStr"/>
       <c r="O187" t="inlineStr"/>
@@ -21419,7 +22551,11 @@
           <t>https://en.wikipedia.org/wiki/6abc_Dunkin%27_Thanksgiving_Day_Parade</t>
         </is>
       </c>
-      <c r="T187" s="2" t="inlineStr"/>
+      <c r="T187" s="2" t="inlineStr">
+        <is>
+          <t>no website in NCES</t>
+        </is>
+      </c>
     </row>
     <row r="188">
       <c r="A188" t="inlineStr">
@@ -21462,17 +22598,32 @@
         <v>2018</v>
       </c>
       <c r="J188" t="inlineStr"/>
-      <c r="K188" t="inlineStr"/>
-      <c r="L188" t="inlineStr"/>
-      <c r="M188" t="inlineStr"/>
-      <c r="N188" t="inlineStr"/>
+      <c r="K188" t="inlineStr">
+        <is>
+          <t>Norwalk School District</t>
+        </is>
+      </c>
+      <c r="L188" t="n">
+        <v>1766</v>
+      </c>
+      <c r="M188" t="inlineStr">
+        <is>
+          <t>http://bmhs.norwalkps.org</t>
+        </is>
+      </c>
+      <c r="N188" t="inlineStr">
+        <is>
+          <t>http://bmhs.norwalkps.org/activities/music-department</t>
+        </is>
+      </c>
       <c r="O188" t="inlineStr"/>
       <c r="P188" t="inlineStr"/>
       <c r="Q188" t="inlineStr"/>
       <c r="R188" t="inlineStr"/>
       <c r="S188" s="2" t="inlineStr">
         <is>
-          <t>https://en.wikipedia.org/wiki/6abc_Dunkin%27_Thanksgiving_Day_Parade</t>
+          <t>https://en.wikipedia.org/wiki/6abc_Dunkin%27_Thanksgiving_Day_Parade
+http://bmhs.norwalkps.org/activities/music-department</t>
         </is>
       </c>
       <c r="T188" s="2" t="inlineStr"/>
@@ -21527,7 +22678,11 @@
           <t>https://en.wikipedia.org/wiki/6abc_Dunkin%27_Thanksgiving_Day_Parade</t>
         </is>
       </c>
-      <c r="T189" s="2" t="inlineStr"/>
+      <c r="T189" s="2" t="inlineStr">
+        <is>
+          <t>nces: no match</t>
+        </is>
+      </c>
     </row>
     <row r="190">
       <c r="A190" t="inlineStr">
@@ -21566,8 +22721,14 @@
         <v>2018</v>
       </c>
       <c r="J190" t="inlineStr"/>
-      <c r="K190" t="inlineStr"/>
-      <c r="L190" t="inlineStr"/>
+      <c r="K190" t="inlineStr">
+        <is>
+          <t>Dublin City</t>
+        </is>
+      </c>
+      <c r="L190" t="n">
+        <v>1878</v>
+      </c>
       <c r="M190" t="inlineStr"/>
       <c r="N190" t="inlineStr"/>
       <c r="O190" t="inlineStr"/>
@@ -21579,7 +22740,11 @@
           <t>https://en.wikipedia.org/wiki/6abc_Dunkin%27_Thanksgiving_Day_Parade</t>
         </is>
       </c>
-      <c r="T190" s="2" t="inlineStr"/>
+      <c r="T190" s="2" t="inlineStr">
+        <is>
+          <t>nces: matched 'Dublin Coffman High School' (0.92); no website in NCES</t>
+        </is>
+      </c>
     </row>
     <row r="191">
       <c r="A191" t="inlineStr">
@@ -21622,8 +22787,14 @@
         <v>2018</v>
       </c>
       <c r="J191" t="inlineStr"/>
-      <c r="K191" t="inlineStr"/>
-      <c r="L191" t="inlineStr"/>
+      <c r="K191" t="inlineStr">
+        <is>
+          <t>Dublin City</t>
+        </is>
+      </c>
+      <c r="L191" t="n">
+        <v>2009</v>
+      </c>
       <c r="M191" t="inlineStr"/>
       <c r="N191" t="inlineStr"/>
       <c r="O191" t="inlineStr"/>
@@ -21635,7 +22806,11 @@
           <t>https://en.wikipedia.org/wiki/6abc_Dunkin%27_Thanksgiving_Day_Parade</t>
         </is>
       </c>
-      <c r="T191" s="2" t="inlineStr"/>
+      <c r="T191" s="2" t="inlineStr">
+        <is>
+          <t>no website in NCES</t>
+        </is>
+      </c>
     </row>
     <row r="192">
       <c r="A192" t="inlineStr">
@@ -21674,8 +22849,14 @@
         <v>2018</v>
       </c>
       <c r="J192" t="inlineStr"/>
-      <c r="K192" t="inlineStr"/>
-      <c r="L192" t="inlineStr"/>
+      <c r="K192" t="inlineStr">
+        <is>
+          <t>Dublin City</t>
+        </is>
+      </c>
+      <c r="L192" t="n">
+        <v>1408</v>
+      </c>
       <c r="M192" t="inlineStr"/>
       <c r="N192" t="inlineStr"/>
       <c r="O192" t="inlineStr"/>
@@ -21687,7 +22868,11 @@
           <t>https://en.wikipedia.org/wiki/6abc_Dunkin%27_Thanksgiving_Day_Parade</t>
         </is>
       </c>
-      <c r="T192" s="2" t="inlineStr"/>
+      <c r="T192" s="2" t="inlineStr">
+        <is>
+          <t>nces: matched 'Dublin Scioto High School' (0.92); no website in NCES</t>
+        </is>
+      </c>
     </row>
     <row r="193">
       <c r="A193" t="inlineStr">
@@ -21730,9 +22915,19 @@
         <v>2016</v>
       </c>
       <c r="J193" t="inlineStr"/>
-      <c r="K193" t="inlineStr"/>
-      <c r="L193" t="inlineStr"/>
-      <c r="M193" t="inlineStr"/>
+      <c r="K193" t="inlineStr">
+        <is>
+          <t>Englewood Public School District</t>
+        </is>
+      </c>
+      <c r="L193" t="n">
+        <v>1078</v>
+      </c>
+      <c r="M193" t="inlineStr">
+        <is>
+          <t>http://dmhs.epsd.org</t>
+        </is>
+      </c>
       <c r="N193" t="inlineStr"/>
       <c r="O193" t="inlineStr"/>
       <c r="P193" t="inlineStr"/>
@@ -21743,7 +22938,11 @@
           <t>https://en.wikipedia.org/wiki/6abc_Dunkin%27_Thanksgiving_Day_Parade</t>
         </is>
       </c>
-      <c r="T193" s="2" t="inlineStr"/>
+      <c r="T193" s="2" t="inlineStr">
+        <is>
+          <t>nces: matched 'Dwight Morrow High School/Academies@Englewood' (0.92); no band page found in 1 pages crawled</t>
+        </is>
+      </c>
     </row>
     <row r="194">
       <c r="A194" t="inlineStr">
@@ -21782,9 +22981,19 @@
         <v>2019</v>
       </c>
       <c r="J194" t="inlineStr"/>
-      <c r="K194" t="inlineStr"/>
-      <c r="L194" t="inlineStr"/>
-      <c r="M194" t="inlineStr"/>
+      <c r="K194" t="inlineStr">
+        <is>
+          <t>Bethlehem Area SD</t>
+        </is>
+      </c>
+      <c r="L194" t="n">
+        <v>1813</v>
+      </c>
+      <c r="M194" t="inlineStr">
+        <is>
+          <t>http://www.beth.k12.pa.us</t>
+        </is>
+      </c>
       <c r="N194" t="inlineStr"/>
       <c r="O194" t="inlineStr"/>
       <c r="P194" t="inlineStr"/>
@@ -21795,7 +23004,11 @@
           <t>https://en.wikipedia.org/wiki/6abc_Dunkin%27_Thanksgiving_Day_Parade</t>
         </is>
       </c>
-      <c r="T194" s="2" t="inlineStr"/>
+      <c r="T194" s="2" t="inlineStr">
+        <is>
+          <t>nces: matched 'Freedom HS' (0.92); no band page found in 2 pages crawled</t>
+        </is>
+      </c>
     </row>
     <row r="195">
       <c r="A195" t="inlineStr">
@@ -21841,7 +23054,7 @@
       </c>
       <c r="T195" s="2" t="inlineStr">
         <is>
-          <t>state unknown: source lists no location</t>
+          <t>state unknown: source lists no location; nces: skipped (state unknown)</t>
         </is>
       </c>
     </row>
@@ -21895,7 +23108,11 @@
           <t>https://en.wikipedia.org/wiki/6abc_Dunkin%27_Thanksgiving_Day_Parade</t>
         </is>
       </c>
-      <c r="T196" s="2" t="inlineStr"/>
+      <c r="T196" s="2" t="inlineStr">
+        <is>
+          <t>nces: low-confidence match 'Jackson High School, Jackson' (0.80); other candidates: Jackson High School (Massillon), Jackson Center High School (Jackson Center); no website in NCES</t>
+        </is>
+      </c>
     </row>
     <row r="197">
       <c r="A197" t="inlineStr">
@@ -21934,9 +23151,19 @@
         <v>2015</v>
       </c>
       <c r="J197" t="inlineStr"/>
-      <c r="K197" t="inlineStr"/>
-      <c r="L197" t="inlineStr"/>
-      <c r="M197" t="inlineStr"/>
+      <c r="K197" t="inlineStr">
+        <is>
+          <t>Jackson Township School District</t>
+        </is>
+      </c>
+      <c r="L197" t="n">
+        <v>1496</v>
+      </c>
+      <c r="M197" t="inlineStr">
+        <is>
+          <t>http://www.jacksonsd.org/Memorial</t>
+        </is>
+      </c>
       <c r="N197" t="inlineStr"/>
       <c r="O197" t="inlineStr"/>
       <c r="P197" t="inlineStr"/>
@@ -21947,7 +23174,11 @@
           <t>https://en.wikipedia.org/wiki/6abc_Dunkin%27_Thanksgiving_Day_Parade</t>
         </is>
       </c>
-      <c r="T197" s="2" t="inlineStr"/>
+      <c r="T197" s="2" t="inlineStr">
+        <is>
+          <t>nces: matched 'Jackson Memorial High School' (0.92); site crawl blocked: HTTP 404 for http://www.jacksonsd.org/Memorial</t>
+        </is>
+      </c>
     </row>
     <row r="198">
       <c r="A198" t="inlineStr">
@@ -21990,8 +23221,14 @@
         <v>2016</v>
       </c>
       <c r="J198" t="inlineStr"/>
-      <c r="K198" t="inlineStr"/>
-      <c r="L198" t="inlineStr"/>
+      <c r="K198" t="inlineStr">
+        <is>
+          <t>Jonathan Alder Local</t>
+        </is>
+      </c>
+      <c r="L198" t="n">
+        <v>671</v>
+      </c>
       <c r="M198" t="inlineStr"/>
       <c r="N198" t="inlineStr"/>
       <c r="O198" t="inlineStr"/>
@@ -22003,7 +23240,11 @@
           <t>https://en.wikipedia.org/wiki/6abc_Dunkin%27_Thanksgiving_Day_Parade</t>
         </is>
       </c>
-      <c r="T198" s="2" t="inlineStr"/>
+      <c r="T198" s="2" t="inlineStr">
+        <is>
+          <t>nces: matched 'Jonathan Alder High School' (0.93); no website in NCES</t>
+        </is>
+      </c>
     </row>
     <row r="199">
       <c r="A199" t="inlineStr">
@@ -22042,9 +23283,19 @@
         <v>2019</v>
       </c>
       <c r="J199" t="inlineStr"/>
-      <c r="K199" t="inlineStr"/>
-      <c r="L199" t="inlineStr"/>
-      <c r="M199" t="inlineStr"/>
+      <c r="K199" t="inlineStr">
+        <is>
+          <t>Kingsway Regional School District</t>
+        </is>
+      </c>
+      <c r="L199" t="n">
+        <v>1984</v>
+      </c>
+      <c r="M199" t="inlineStr">
+        <is>
+          <t>http://www.krsd.org</t>
+        </is>
+      </c>
       <c r="N199" t="inlineStr"/>
       <c r="O199" t="inlineStr"/>
       <c r="P199" t="inlineStr"/>
@@ -22055,7 +23306,11 @@
           <t>https://en.wikipedia.org/wiki/6abc_Dunkin%27_Thanksgiving_Day_Parade</t>
         </is>
       </c>
-      <c r="T199" s="2" t="inlineStr"/>
+      <c r="T199" s="2" t="inlineStr">
+        <is>
+          <t>nces: matched 'Kingsway Regional High School' (0.92); no band page found in 7 pages crawled</t>
+        </is>
+      </c>
     </row>
     <row r="200">
       <c r="A200" t="inlineStr">
@@ -22111,7 +23366,11 @@
           <t>https://en.wikipedia.org/wiki/6abc_Dunkin%27_Thanksgiving_Day_Parade</t>
         </is>
       </c>
-      <c r="T200" s="2" t="inlineStr"/>
+      <c r="T200" s="2" t="inlineStr">
+        <is>
+          <t>nces: no match</t>
+        </is>
+      </c>
     </row>
     <row r="201">
       <c r="A201" t="inlineStr">
@@ -22154,8 +23413,14 @@
         <v>2015</v>
       </c>
       <c r="J201" t="inlineStr"/>
-      <c r="K201" t="inlineStr"/>
-      <c r="L201" t="inlineStr"/>
+      <c r="K201" t="inlineStr">
+        <is>
+          <t>LaPorte Community School Corp</t>
+        </is>
+      </c>
+      <c r="L201" t="n">
+        <v>1851</v>
+      </c>
       <c r="M201" t="inlineStr"/>
       <c r="N201" t="inlineStr"/>
       <c r="O201" t="inlineStr"/>
@@ -22167,7 +23432,11 @@
           <t>https://en.wikipedia.org/wiki/6abc_Dunkin%27_Thanksgiving_Day_Parade</t>
         </is>
       </c>
-      <c r="T201" s="2" t="inlineStr"/>
+      <c r="T201" s="2" t="inlineStr">
+        <is>
+          <t>no website in NCES</t>
+        </is>
+      </c>
     </row>
     <row r="202">
       <c r="A202" t="inlineStr">
@@ -22210,9 +23479,19 @@
         <v>2018</v>
       </c>
       <c r="J202" t="inlineStr"/>
-      <c r="K202" t="inlineStr"/>
-      <c r="L202" t="inlineStr"/>
-      <c r="M202" t="inlineStr"/>
+      <c r="K202" t="inlineStr">
+        <is>
+          <t>Lenape Regional High School District</t>
+        </is>
+      </c>
+      <c r="L202" t="n">
+        <v>1922</v>
+      </c>
+      <c r="M202" t="inlineStr">
+        <is>
+          <t>http://www.lrhsd.org/Domain/119</t>
+        </is>
+      </c>
       <c r="N202" t="inlineStr"/>
       <c r="O202" t="inlineStr"/>
       <c r="P202" t="inlineStr"/>
@@ -22223,7 +23502,11 @@
           <t>https://en.wikipedia.org/wiki/6abc_Dunkin%27_Thanksgiving_Day_Parade</t>
         </is>
       </c>
-      <c r="T202" s="2" t="inlineStr"/>
+      <c r="T202" s="2" t="inlineStr">
+        <is>
+          <t>nces: matched 'Lenape High School' (0.92); site crawl blocked: HTTP 404 for http://www.lrhsd.org/Domain/119</t>
+        </is>
+      </c>
     </row>
     <row r="203">
       <c r="A203" t="inlineStr">
@@ -22266,9 +23549,19 @@
         <v>2018</v>
       </c>
       <c r="J203" t="inlineStr"/>
-      <c r="K203" t="inlineStr"/>
-      <c r="L203" t="inlineStr"/>
-      <c r="M203" t="inlineStr"/>
+      <c r="K203" t="inlineStr">
+        <is>
+          <t>Muskego-Norway School District</t>
+        </is>
+      </c>
+      <c r="L203" t="n">
+        <v>1651</v>
+      </c>
+      <c r="M203" t="inlineStr">
+        <is>
+          <t>http://www.muskegonorway.org</t>
+        </is>
+      </c>
       <c r="N203" t="inlineStr"/>
       <c r="O203" t="inlineStr"/>
       <c r="P203" t="inlineStr"/>
@@ -22279,7 +23572,11 @@
           <t>https://en.wikipedia.org/wiki/6abc_Dunkin%27_Thanksgiving_Day_Parade</t>
         </is>
       </c>
-      <c r="T203" s="2" t="inlineStr"/>
+      <c r="T203" s="2" t="inlineStr">
+        <is>
+          <t>nces: matched 'Muskego High' (0.92); no band page found in 4 pages crawled</t>
+        </is>
+      </c>
     </row>
     <row r="204">
       <c r="A204" t="inlineStr">
@@ -22322,8 +23619,14 @@
         <v>2016</v>
       </c>
       <c r="J204" t="inlineStr"/>
-      <c r="K204" t="inlineStr"/>
-      <c r="L204" t="inlineStr"/>
+      <c r="K204" t="inlineStr">
+        <is>
+          <t>Wa-Nee Community Schools</t>
+        </is>
+      </c>
+      <c r="L204" t="n">
+        <v>875</v>
+      </c>
       <c r="M204" t="inlineStr"/>
       <c r="N204" t="inlineStr"/>
       <c r="O204" t="inlineStr"/>
@@ -22335,7 +23638,11 @@
           <t>https://en.wikipedia.org/wiki/6abc_Dunkin%27_Thanksgiving_Day_Parade</t>
         </is>
       </c>
-      <c r="T204" s="2" t="inlineStr"/>
+      <c r="T204" s="2" t="inlineStr">
+        <is>
+          <t>nces: matched 'North Wood High School' (0.95); no website in NCES</t>
+        </is>
+      </c>
     </row>
     <row r="205">
       <c r="A205" t="inlineStr">
@@ -22378,8 +23685,14 @@
         <v>2018</v>
       </c>
       <c r="J205" t="inlineStr"/>
-      <c r="K205" t="inlineStr"/>
-      <c r="L205" t="inlineStr"/>
+      <c r="K205" t="inlineStr">
+        <is>
+          <t>Hawaii Department of Education</t>
+        </is>
+      </c>
+      <c r="L205" t="n">
+        <v>1418</v>
+      </c>
       <c r="M205" t="inlineStr"/>
       <c r="N205" t="inlineStr"/>
       <c r="O205" t="inlineStr"/>
@@ -22391,7 +23704,11 @@
           <t>https://en.wikipedia.org/wiki/6abc_Dunkin%27_Thanksgiving_Day_Parade</t>
         </is>
       </c>
-      <c r="T205" s="2" t="inlineStr"/>
+      <c r="T205" s="2" t="inlineStr">
+        <is>
+          <t>no website in NCES</t>
+        </is>
+      </c>
     </row>
     <row r="206">
       <c r="A206" t="inlineStr">
@@ -22434,8 +23751,14 @@
         <v>2015</v>
       </c>
       <c r="J206" t="inlineStr"/>
-      <c r="K206" t="inlineStr"/>
-      <c r="L206" t="inlineStr"/>
+      <c r="K206" t="inlineStr">
+        <is>
+          <t>South Madison Com Sch Corp</t>
+        </is>
+      </c>
+      <c r="L206" t="n">
+        <v>1353</v>
+      </c>
       <c r="M206" t="inlineStr"/>
       <c r="N206" t="inlineStr"/>
       <c r="O206" t="inlineStr"/>
@@ -22447,7 +23770,11 @@
           <t>https://en.wikipedia.org/wiki/6abc_Dunkin%27_Thanksgiving_Day_Parade</t>
         </is>
       </c>
-      <c r="T206" s="2" t="inlineStr"/>
+      <c r="T206" s="2" t="inlineStr">
+        <is>
+          <t>no website in NCES</t>
+        </is>
+      </c>
     </row>
     <row r="207">
       <c r="A207" t="inlineStr">
@@ -22499,7 +23826,11 @@
           <t>https://en.wikipedia.org/wiki/6abc_Dunkin%27_Thanksgiving_Day_Parade</t>
         </is>
       </c>
-      <c r="T207" s="2" t="inlineStr"/>
+      <c r="T207" s="2" t="inlineStr">
+        <is>
+          <t>nces: no match</t>
+        </is>
+      </c>
     </row>
     <row r="208">
       <c r="A208" t="inlineStr">
@@ -22542,8 +23873,14 @@
         <v>2019</v>
       </c>
       <c r="J208" t="inlineStr"/>
-      <c r="K208" t="inlineStr"/>
-      <c r="L208" t="inlineStr"/>
+      <c r="K208" t="inlineStr">
+        <is>
+          <t>Twin Lakes School Corp</t>
+        </is>
+      </c>
+      <c r="L208" t="n">
+        <v>663</v>
+      </c>
       <c r="M208" t="inlineStr"/>
       <c r="N208" t="inlineStr"/>
       <c r="O208" t="inlineStr"/>
@@ -22555,7 +23892,11 @@
           <t>https://en.wikipedia.org/wiki/6abc_Dunkin%27_Thanksgiving_Day_Parade</t>
         </is>
       </c>
-      <c r="T208" s="2" t="inlineStr"/>
+      <c r="T208" s="2" t="inlineStr">
+        <is>
+          <t>no website in NCES</t>
+        </is>
+      </c>
     </row>
     <row r="209">
       <c r="A209" t="inlineStr">
@@ -22598,8 +23939,14 @@
         <v>2016</v>
       </c>
       <c r="J209" t="inlineStr"/>
-      <c r="K209" t="inlineStr"/>
-      <c r="L209" t="inlineStr"/>
+      <c r="K209" t="inlineStr">
+        <is>
+          <t>Randolph Central School Corp</t>
+        </is>
+      </c>
+      <c r="L209" t="n">
+        <v>408</v>
+      </c>
       <c r="M209" t="inlineStr"/>
       <c r="N209" t="inlineStr"/>
       <c r="O209" t="inlineStr"/>
@@ -22611,7 +23958,11 @@
           <t>https://en.wikipedia.org/wiki/6abc_Dunkin%27_Thanksgiving_Day_Parade</t>
         </is>
       </c>
-      <c r="T209" s="2" t="inlineStr"/>
+      <c r="T209" s="2" t="inlineStr">
+        <is>
+          <t>no website in NCES</t>
+        </is>
+      </c>
     </row>
   </sheetData>
   <autoFilter ref="A1:T209"/>

</xml_diff>

<commit_message>
Drop a stale Middle level on rebuild when the school name does not say middle
Co-Authored-By: Claude Fable 5.1 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_014hr17qS7ZCdG5VTCbF27VQ
</commit_message>
<xml_diff>
--- a/data/final/prospects.xlsx
+++ b/data/final/prospects.xlsx
@@ -6707,11 +6707,7 @@
           <t>GA</t>
         </is>
       </c>
-      <c r="G37" t="inlineStr">
-        <is>
-          <t>Middle</t>
-        </is>
-      </c>
+      <c r="G37" t="inlineStr"/>
       <c r="H37" s="2" t="inlineStr">
         <is>
           <t>Rose 2017</t>
@@ -11815,11 +11811,7 @@
           <t>GA</t>
         </is>
       </c>
-      <c r="G12" t="inlineStr">
-        <is>
-          <t>Middle</t>
-        </is>
-      </c>
+      <c r="G12" t="inlineStr"/>
       <c r="H12" s="2" t="inlineStr">
         <is>
           <t>Rose 2017</t>
@@ -20545,11 +20537,7 @@
           <t>GA</t>
         </is>
       </c>
-      <c r="G87" t="inlineStr">
-        <is>
-          <t>Middle</t>
-        </is>
-      </c>
+      <c r="G87" t="inlineStr"/>
       <c r="H87" s="2" t="inlineStr">
         <is>
           <t>Rose 2017</t>

</xml_diff>

<commit_message>
QA pass over prefix-boosted NCES matches: one corrected, one withdrawn, boost tightened
scripts/qa.py (new) re-checks every NCES match noted at 0.92. Olentangy Orange
High School (OH) had been matched to "Olentangy High School"; NCES lists it as
"Orange High School" in the same district, so the row is re-pointed (enrollment
1721 -> 1967). Downingtown High School (PA) is withdrawn as ambiguous (East
Campus, West Campus, STEM Academy): district kept, enrollment blanked, candidates
noted. The other 40 prefix matches were benign.

enrich.match_nces no longer applies the prefix boost when the row's extra word
names another school in the state, or when several NCES names extend the prefix.
Tests: 57 pass. Docs and CHANGELOG updated; scores and exports rebuilt.

Co-Authored-By: Claude Fable 5.1 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_0192hWqZ8pcqLVQqxHYF7nEh
</commit_message>
<xml_diff>
--- a/data/final/prospects.xlsx
+++ b/data/final/prospects.xlsx
@@ -6791,7 +6791,7 @@
         </is>
       </c>
       <c r="M35" t="n">
-        <v>1721</v>
+        <v>1967</v>
       </c>
       <c r="N35" t="inlineStr"/>
       <c r="O35" t="inlineStr"/>
@@ -6807,7 +6807,7 @@
       </c>
       <c r="U35" s="2" t="inlineStr">
         <is>
-          <t>nces: matched 'Olentangy High School' (0.92); no website in NCES; search: Google knowledge panel is in a county/township, not Lewis Center, and no NCES schools carry this name in OH; not used</t>
+          <t>nces: prefix match 'Olentangy High School' corrected to 'Orange High School' (same district; name carries the row's word); no website in NCES; search: Google knowledge panel is in a county/township, not Lewis Center, and no NCES schools carry this name in OH; not used</t>
         </is>
       </c>
     </row>
@@ -7008,9 +7008,7 @@
           <t>Downingtown Area SD</t>
         </is>
       </c>
-      <c r="M38" t="n">
-        <v>1808</v>
-      </c>
+      <c r="M38" t="inlineStr"/>
       <c r="N38" t="inlineStr"/>
       <c r="O38" t="inlineStr"/>
       <c r="P38" t="inlineStr"/>
@@ -7024,7 +7022,7 @@
       </c>
       <c r="U38" s="2" t="inlineStr">
         <is>
-          <t>nces: matched 'Downingtown HS West Campus' (0.92); no website in NCES; search: no school site found</t>
+          <t>nces: prefix match 'Downingtown HS West Campus' withdrawn as ambiguous; candidates: Downingtown HS East Campus (Exton), Downingtown HS West Campus (Downingtown), Downingtown STEM Academy (Downingtown); no website in NCES; search: no school site found</t>
         </is>
       </c>
     </row>
@@ -12352,9 +12350,7 @@
           <t>Downingtown Area SD</t>
         </is>
       </c>
-      <c r="M14" t="n">
-        <v>1808</v>
-      </c>
+      <c r="M14" t="inlineStr"/>
       <c r="N14" t="inlineStr"/>
       <c r="O14" t="inlineStr"/>
       <c r="P14" t="inlineStr"/>
@@ -12368,7 +12364,7 @@
       </c>
       <c r="U14" s="2" t="inlineStr">
         <is>
-          <t>nces: matched 'Downingtown HS West Campus' (0.92); no website in NCES; search: no school site found</t>
+          <t>nces: prefix match 'Downingtown HS West Campus' withdrawn as ambiguous; candidates: Downingtown HS East Campus (Exton), Downingtown HS West Campus (Downingtown), Downingtown STEM Academy (Downingtown); no website in NCES; search: no school site found</t>
         </is>
       </c>
     </row>
@@ -21476,7 +21472,7 @@
         </is>
       </c>
       <c r="M85" t="n">
-        <v>1721</v>
+        <v>1967</v>
       </c>
       <c r="N85" t="inlineStr"/>
       <c r="O85" t="inlineStr"/>
@@ -21492,7 +21488,7 @@
       </c>
       <c r="U85" s="2" t="inlineStr">
         <is>
-          <t>nces: matched 'Olentangy High School' (0.92); no website in NCES; search: Google knowledge panel is in a county/township, not Lewis Center, and no NCES schools carry this name in OH; not used</t>
+          <t>nces: prefix match 'Olentangy High School' corrected to 'Orange High School' (same district; name carries the row's word); no website in NCES; search: Google knowledge panel is in a county/township, not Lewis Center, and no NCES schools carry this name in OH; not used</t>
         </is>
       </c>
     </row>
@@ -21693,9 +21689,7 @@
           <t>Downingtown Area SD</t>
         </is>
       </c>
-      <c r="M88" t="n">
-        <v>1808</v>
-      </c>
+      <c r="M88" t="inlineStr"/>
       <c r="N88" t="inlineStr"/>
       <c r="O88" t="inlineStr"/>
       <c r="P88" t="inlineStr"/>
@@ -21709,7 +21703,7 @@
       </c>
       <c r="U88" s="2" t="inlineStr">
         <is>
-          <t>nces: matched 'Downingtown HS West Campus' (0.92); no website in NCES; search: no school site found</t>
+          <t>nces: prefix match 'Downingtown HS West Campus' withdrawn as ambiguous; candidates: Downingtown HS East Campus (Exton), Downingtown HS West Campus (Downingtown), Downingtown STEM Academy (Downingtown); no website in NCES; search: no school site found</t>
         </is>
       </c>
     </row>

</xml_diff>